<commit_message>
Revert "Merge remote-tracking branch 'origin/Develop' into feature/Object"
This reverts commit b8be80b274d255db894f10cfcb23fc05a5837277, reversing
changes made to 8e1d4309fe6a5a017622e9cda4e2c324031ac1a4.
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/ItemData.xlsx
+++ b/JsonConverter/ExcelFiles/ItemData.xlsx
@@ -1,28 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <workbookPr/>
-  <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9000"/>
-  </bookViews>
   <sheets>
-    <sheet name="ItemData" sheetId="1" r:id="rId1"/>
+    <sheet state="visible" name="ItemData" sheetId="1" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr/>
 </workbook>
 </file>
 
@@ -167,203 +151,41 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="25">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <fonts count="5">
     <font>
-      <sz val="10"/>
+      <sz val="10.0"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
+      <sz val="10.0"/>
       <color rgb="FF000000"/>
       <name val="&quot;맑은 고딕&quot;"/>
-      <charset val="134"/>
     </font>
     <font>
-      <sz val="10"/>
+      <sz val="10.0"/>
       <color rgb="FF000000"/>
       <name val="Malgun Gothic"/>
-      <charset val="134"/>
     </font>
     <font>
-      <sz val="10"/>
+      <sz val="10.0"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
-      <charset val="134"/>
     </font>
     <font>
-      <sz val="11"/>
+      <sz val="11.0"/>
       <color rgb="FF008000"/>
       <name val="&quot;맑은 고딕&quot;"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="35">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="gray125"/>
+      <patternFill patternType="lightGray"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -377,201 +199,9 @@
         <bgColor rgb="FFD2F2DB"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="10">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
+  <borders count="2">
+    <border/>
     <border>
       <left style="thin">
         <color rgb="FF000000"/>
@@ -585,545 +215,60 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="49">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
+  <cellStyleXfs count="1">
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+  </cellStyleXfs>
+  <cellXfs count="10">
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
+    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" vertical="bottom"/>
     </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
+    <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="177" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
+    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="42" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
+    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
+    <xf borderId="1" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
+    <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
+    <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
+    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-  </cellStyleXfs>
-  <cellXfs count="7">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="right" readingOrder="0" vertical="bottom"/>
     </xf>
   </cellXfs>
-  <cellStyles count="49">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Currency" xfId="2" builtinId="4"/>
-    <cellStyle name="Percent" xfId="3" builtinId="5"/>
-    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
-    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Link" xfId="6" builtinId="8"/>
-    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
-    <cellStyle name="Note" xfId="8" builtinId="10"/>
-    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
-    <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
-    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
-    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
-    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
-    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
-    <cellStyle name="Input" xfId="16" builtinId="20"/>
-    <cellStyle name="Output" xfId="17" builtinId="21"/>
-    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
-    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
-    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
-    <cellStyle name="Total" xfId="21" builtinId="25"/>
-    <cellStyle name="Good" xfId="22" builtinId="26"/>
-    <cellStyle name="Bad" xfId="23" builtinId="27"/>
-    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
-    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
-    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
-    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
-    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
-    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
-    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
+  <cellStyles count="1">
+    <cellStyle xfId="0" name="Normal" builtinId="0"/>
   </cellStyles>
-  <dxfs count="17">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <border>
-        <top style="double">
-          <color theme="4"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4"/>
-          <bgColor theme="4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <border>
-        <left style="thin">
-          <color theme="4"/>
-        </left>
-        <right style="thin">
-          <color theme="4"/>
-        </right>
-        <top style="thin">
-          <color theme="4"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4"/>
-        </bottom>
-        <horizontal style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <border>
-        <top style="thin">
-          <color theme="4"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-  </dxfs>
-  <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
-    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{59DB682C-5494-4EDE-A608-00C9E5F0F923}">
-      <tableStyleElement type="wholeTable" dxfId="6"/>
-      <tableStyleElement type="headerRow" dxfId="5"/>
-      <tableStyleElement type="totalRow" dxfId="4"/>
-      <tableStyleElement type="firstColumn" dxfId="3"/>
-      <tableStyleElement type="lastColumn" dxfId="2"/>
-      <tableStyleElement type="firstRowStripe" dxfId="1"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="0"/>
-    </tableStyle>
-    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{267968C8-6FFD-4C36-ACC1-9EA1FD1885CA}">
-      <tableStyleElement type="headerRow" dxfId="16"/>
-      <tableStyleElement type="totalRow" dxfId="15"/>
-      <tableStyleElement type="firstRowStripe" dxfId="14"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="13"/>
-      <tableStyleElement type="firstSubtotalRow" dxfId="12"/>
-      <tableStyleElement type="secondSubtotalRow" dxfId="11"/>
-      <tableStyleElement type="firstRowSubheading" dxfId="10"/>
-      <tableStyleElement type="secondRowSubheading" dxfId="9"/>
-      <tableStyleElement type="pageFieldLabels" dxfId="8"/>
-      <tableStyleElement type="pageFieldValues" dxfId="7"/>
-    </tableStyle>
-  </tableStyles>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <dxfs count="0"/>
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -1313,35 +458,34 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
+    <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z1000"/>
-  <sheetFormatPr defaultColWidth="12.6296296296296" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="19.3796296296296" customWidth="1"/>
-    <col min="2" max="2" width="17.1296296296296" customWidth="1"/>
-    <col min="3" max="3" width="44.3796296296296" customWidth="1"/>
-    <col min="4" max="4" width="17.75" customWidth="1"/>
-    <col min="5" max="5" width="19.75" customWidth="1"/>
-    <col min="6" max="6" width="13.25" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="27.1296296296296" customWidth="1"/>
-    <col min="9" max="9" width="28.25" customWidth="1"/>
-    <col min="10" max="10" width="14.6296296296296" customWidth="1"/>
-    <col min="11" max="11" width="12.8796296296296" customWidth="1"/>
-    <col min="12" max="12" width="11" customWidth="1"/>
-    <col min="13" max="13" width="17.3796296296296" customWidth="1"/>
-    <col min="14" max="26" width="11" customWidth="1"/>
+    <col customWidth="1" min="1" max="1" width="19.38"/>
+    <col customWidth="1" min="2" max="2" width="17.13"/>
+    <col customWidth="1" min="3" max="3" width="44.38"/>
+    <col customWidth="1" min="4" max="4" width="17.75"/>
+    <col customWidth="1" min="5" max="5" width="19.75"/>
+    <col customWidth="1" min="6" max="6" width="13.25"/>
+    <col customWidth="1" min="7" max="7" width="11.0"/>
+    <col customWidth="1" min="8" max="8" width="27.13"/>
+    <col customWidth="1" min="9" max="9" width="28.25"/>
+    <col customWidth="1" min="10" max="10" width="14.63"/>
+    <col customWidth="1" min="11" max="11" width="12.88"/>
+    <col customWidth="1" min="12" max="12" width="11.0"/>
+    <col customWidth="1" min="13" max="13" width="17.38"/>
+    <col customWidth="1" min="14" max="26" width="11.0"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1" spans="1:26">
+    <row r="1" ht="15.75" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1369,16 +513,16 @@
       <c r="I1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="L1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="M1" s="4" t="s">
         <v>12</v>
       </c>
       <c r="N1" s="3"/>
@@ -1395,7 +539,7 @@
       <c r="Y1" s="3"/>
       <c r="Z1" s="3"/>
     </row>
-    <row r="2" ht="13.2" spans="1:26">
+    <row r="2">
       <c r="A2" s="1" t="s">
         <v>13</v>
       </c>
@@ -1423,16 +567,16 @@
       <c r="I2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="J2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="K2" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="L2" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="M2" s="4" t="s">
         <v>16</v>
       </c>
       <c r="N2" s="3"/>
@@ -1449,81 +593,81 @@
       <c r="Y2" s="3"/>
       <c r="Z2" s="3"/>
     </row>
-    <row r="3" ht="15.75" customHeight="1" spans="1:26">
-      <c r="A3" s="4" t="s">
+    <row r="3" ht="15.75" customHeight="1">
+      <c r="A3" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="H3" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="I3" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="J3" s="5" t="s">
+      <c r="J3" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="K3" s="5" t="s">
+      <c r="K3" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="L3" s="5" t="s">
+      <c r="L3" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="M3" s="5" t="s">
+      <c r="M3" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="N3" s="5"/>
-      <c r="O3" s="5"/>
-      <c r="P3" s="5"/>
-      <c r="Q3" s="5"/>
-      <c r="R3" s="5"/>
-      <c r="S3" s="5"/>
-      <c r="T3" s="5"/>
-      <c r="U3" s="5"/>
-      <c r="V3" s="5"/>
-      <c r="W3" s="5"/>
-      <c r="X3" s="5"/>
-      <c r="Y3" s="5"/>
-      <c r="Z3" s="5"/>
-    </row>
-    <row r="4" ht="15.75" customHeight="1" spans="1:26">
-      <c r="A4" s="1" t="s">
+      <c r="N3" s="6"/>
+      <c r="O3" s="6"/>
+      <c r="P3" s="6"/>
+      <c r="Q3" s="6"/>
+      <c r="R3" s="6"/>
+      <c r="S3" s="6"/>
+      <c r="T3" s="6"/>
+      <c r="U3" s="6"/>
+      <c r="V3" s="6"/>
+      <c r="W3" s="6"/>
+      <c r="X3" s="6"/>
+      <c r="Y3" s="6"/>
+      <c r="Z3" s="6"/>
+    </row>
+    <row r="4" ht="15.75" customHeight="1">
+      <c r="A4" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="F4" s="6">
-        <v>1</v>
+      <c r="F4" s="9">
+        <v>1.0</v>
       </c>
-      <c r="G4" s="3">
-        <v>100</v>
+      <c r="G4" s="4">
+        <v>100.0</v>
       </c>
       <c r="H4" s="3"/>
       <c r="I4" s="3"/>
@@ -1545,32 +689,32 @@
       <c r="Y4" s="3"/>
       <c r="Z4" s="3"/>
     </row>
-    <row r="5" ht="15.75" customHeight="1" spans="1:26">
-      <c r="A5" s="1" t="s">
+    <row r="5" ht="15.75" customHeight="1">
+      <c r="A5" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="F5" s="3">
-        <v>10</v>
+      <c r="F5" s="4">
+        <v>10.0</v>
       </c>
-      <c r="G5" s="3">
-        <v>30</v>
+      <c r="G5" s="4">
+        <v>30.0</v>
       </c>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
-      <c r="J5" s="3">
-        <v>100</v>
+      <c r="J5" s="4">
+        <v>100.0</v>
       </c>
       <c r="K5" s="3"/>
       <c r="L5" s="3"/>
@@ -1589,39 +733,39 @@
       <c r="Y5" s="3"/>
       <c r="Z5" s="3"/>
     </row>
-    <row r="6" ht="15.75" customHeight="1" spans="1:26">
-      <c r="A6" s="1" t="s">
+    <row r="6" ht="15.75" customHeight="1">
+      <c r="A6" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="F6" s="3">
-        <v>2</v>
+      <c r="F6" s="4">
+        <v>2.0</v>
       </c>
-      <c r="G6" s="3">
-        <v>20</v>
+      <c r="G6" s="4">
+        <v>20.0</v>
       </c>
       <c r="H6" s="3"/>
       <c r="I6" s="3"/>
       <c r="J6" s="3"/>
-      <c r="K6" s="3" t="s">
+      <c r="K6" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="L6" s="3">
-        <v>50</v>
+      <c r="L6" s="4">
+        <v>50.0</v>
       </c>
-      <c r="M6" s="3">
-        <v>0</v>
+      <c r="M6" s="4">
+        <v>0.0</v>
       </c>
       <c r="N6" s="3"/>
       <c r="O6" s="3"/>
@@ -1637,7 +781,7 @@
       <c r="Y6" s="3"/>
       <c r="Z6" s="3"/>
     </row>
-    <row r="7" ht="15.75" customHeight="1" spans="1:26">
+    <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -1665,7 +809,7 @@
       <c r="Y7" s="3"/>
       <c r="Z7" s="3"/>
     </row>
-    <row r="8" ht="15.75" customHeight="1" spans="1:26">
+    <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
@@ -1693,7 +837,7 @@
       <c r="Y8" s="3"/>
       <c r="Z8" s="3"/>
     </row>
-    <row r="9" ht="15.75" customHeight="1" spans="1:26">
+    <row r="9" ht="15.75" customHeight="1">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -1721,7 +865,7 @@
       <c r="Y9" s="3"/>
       <c r="Z9" s="3"/>
     </row>
-    <row r="10" ht="15.75" customHeight="1" spans="1:26">
+    <row r="10" ht="15.75" customHeight="1">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
@@ -1749,7 +893,7 @@
       <c r="Y10" s="3"/>
       <c r="Z10" s="3"/>
     </row>
-    <row r="11" ht="15.75" customHeight="1" spans="1:26">
+    <row r="11" ht="15.75" customHeight="1">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -1777,7 +921,7 @@
       <c r="Y11" s="3"/>
       <c r="Z11" s="3"/>
     </row>
-    <row r="12" ht="15.75" customHeight="1" spans="1:26">
+    <row r="12" ht="15.75" customHeight="1">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
@@ -1805,7 +949,7 @@
       <c r="Y12" s="3"/>
       <c r="Z12" s="3"/>
     </row>
-    <row r="13" ht="15.75" customHeight="1" spans="1:26">
+    <row r="13" ht="15.75" customHeight="1">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -1833,7 +977,7 @@
       <c r="Y13" s="3"/>
       <c r="Z13" s="3"/>
     </row>
-    <row r="14" ht="15.75" customHeight="1" spans="1:26">
+    <row r="14" ht="15.75" customHeight="1">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
@@ -1861,7 +1005,7 @@
       <c r="Y14" s="3"/>
       <c r="Z14" s="3"/>
     </row>
-    <row r="15" ht="15.75" customHeight="1" spans="1:26">
+    <row r="15" ht="15.75" customHeight="1">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -1889,7 +1033,7 @@
       <c r="Y15" s="3"/>
       <c r="Z15" s="3"/>
     </row>
-    <row r="16" ht="15.75" customHeight="1" spans="1:26">
+    <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="3"/>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
@@ -1917,7 +1061,7 @@
       <c r="Y16" s="3"/>
       <c r="Z16" s="3"/>
     </row>
-    <row r="17" ht="15.75" customHeight="1" spans="1:26">
+    <row r="17" ht="15.75" customHeight="1">
       <c r="A17" s="3"/>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -1945,7 +1089,7 @@
       <c r="Y17" s="3"/>
       <c r="Z17" s="3"/>
     </row>
-    <row r="18" ht="15.75" customHeight="1" spans="1:26">
+    <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="3"/>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
@@ -1973,7 +1117,7 @@
       <c r="Y18" s="3"/>
       <c r="Z18" s="3"/>
     </row>
-    <row r="19" ht="15.75" customHeight="1" spans="1:26">
+    <row r="19" ht="15.75" customHeight="1">
       <c r="A19" s="3"/>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
@@ -2001,7 +1145,7 @@
       <c r="Y19" s="3"/>
       <c r="Z19" s="3"/>
     </row>
-    <row r="20" ht="15.75" customHeight="1" spans="1:26">
+    <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="3"/>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
@@ -2029,7 +1173,7 @@
       <c r="Y20" s="3"/>
       <c r="Z20" s="3"/>
     </row>
-    <row r="21" ht="15.75" customHeight="1" spans="1:26">
+    <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="3"/>
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
@@ -2057,7 +1201,7 @@
       <c r="Y21" s="3"/>
       <c r="Z21" s="3"/>
     </row>
-    <row r="22" ht="15.75" customHeight="1" spans="1:26">
+    <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="3"/>
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
@@ -2085,7 +1229,7 @@
       <c r="Y22" s="3"/>
       <c r="Z22" s="3"/>
     </row>
-    <row r="23" ht="15.75" customHeight="1" spans="1:26">
+    <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="3"/>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
@@ -2113,7 +1257,7 @@
       <c r="Y23" s="3"/>
       <c r="Z23" s="3"/>
     </row>
-    <row r="24" ht="15.75" customHeight="1" spans="1:26">
+    <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="3"/>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
@@ -2141,7 +1285,7 @@
       <c r="Y24" s="3"/>
       <c r="Z24" s="3"/>
     </row>
-    <row r="25" ht="15.75" customHeight="1" spans="1:26">
+    <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="3"/>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
@@ -2169,7 +1313,7 @@
       <c r="Y25" s="3"/>
       <c r="Z25" s="3"/>
     </row>
-    <row r="26" ht="15.75" customHeight="1" spans="1:26">
+    <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="3"/>
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
@@ -2197,7 +1341,7 @@
       <c r="Y26" s="3"/>
       <c r="Z26" s="3"/>
     </row>
-    <row r="27" ht="15.75" customHeight="1" spans="1:26">
+    <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="3"/>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
@@ -2225,7 +1369,7 @@
       <c r="Y27" s="3"/>
       <c r="Z27" s="3"/>
     </row>
-    <row r="28" ht="15.75" customHeight="1" spans="1:26">
+    <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="3"/>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
@@ -2253,7 +1397,7 @@
       <c r="Y28" s="3"/>
       <c r="Z28" s="3"/>
     </row>
-    <row r="29" ht="15.75" customHeight="1" spans="1:26">
+    <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="3"/>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
@@ -2281,7 +1425,7 @@
       <c r="Y29" s="3"/>
       <c r="Z29" s="3"/>
     </row>
-    <row r="30" ht="15.75" customHeight="1" spans="1:26">
+    <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="3"/>
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
@@ -2309,7 +1453,7 @@
       <c r="Y30" s="3"/>
       <c r="Z30" s="3"/>
     </row>
-    <row r="31" ht="15.75" customHeight="1" spans="1:26">
+    <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="3"/>
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
@@ -2337,7 +1481,7 @@
       <c r="Y31" s="3"/>
       <c r="Z31" s="3"/>
     </row>
-    <row r="32" ht="15.75" customHeight="1" spans="1:26">
+    <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="3"/>
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
@@ -2365,7 +1509,7 @@
       <c r="Y32" s="3"/>
       <c r="Z32" s="3"/>
     </row>
-    <row r="33" ht="15.75" customHeight="1" spans="1:26">
+    <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="3"/>
       <c r="B33" s="3"/>
       <c r="C33" s="3"/>
@@ -2393,7 +1537,7 @@
       <c r="Y33" s="3"/>
       <c r="Z33" s="3"/>
     </row>
-    <row r="34" ht="15.75" customHeight="1" spans="1:26">
+    <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="3"/>
       <c r="B34" s="3"/>
       <c r="C34" s="3"/>
@@ -2421,7 +1565,7 @@
       <c r="Y34" s="3"/>
       <c r="Z34" s="3"/>
     </row>
-    <row r="35" ht="15.75" customHeight="1" spans="1:26">
+    <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="3"/>
       <c r="B35" s="3"/>
       <c r="C35" s="3"/>
@@ -2449,7 +1593,7 @@
       <c r="Y35" s="3"/>
       <c r="Z35" s="3"/>
     </row>
-    <row r="36" ht="15.75" customHeight="1" spans="1:26">
+    <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="3"/>
       <c r="B36" s="3"/>
       <c r="C36" s="3"/>
@@ -2477,7 +1621,7 @@
       <c r="Y36" s="3"/>
       <c r="Z36" s="3"/>
     </row>
-    <row r="37" ht="15.75" customHeight="1" spans="1:26">
+    <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="3"/>
       <c r="B37" s="3"/>
       <c r="C37" s="3"/>
@@ -2505,7 +1649,7 @@
       <c r="Y37" s="3"/>
       <c r="Z37" s="3"/>
     </row>
-    <row r="38" ht="15.75" customHeight="1" spans="1:26">
+    <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="3"/>
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
@@ -2533,7 +1677,7 @@
       <c r="Y38" s="3"/>
       <c r="Z38" s="3"/>
     </row>
-    <row r="39" ht="15.75" customHeight="1" spans="1:26">
+    <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="3"/>
       <c r="B39" s="3"/>
       <c r="C39" s="3"/>
@@ -2561,7 +1705,7 @@
       <c r="Y39" s="3"/>
       <c r="Z39" s="3"/>
     </row>
-    <row r="40" ht="15.75" customHeight="1" spans="1:26">
+    <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="3"/>
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
@@ -2589,7 +1733,7 @@
       <c r="Y40" s="3"/>
       <c r="Z40" s="3"/>
     </row>
-    <row r="41" ht="15.75" customHeight="1" spans="1:26">
+    <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="3"/>
       <c r="B41" s="3"/>
       <c r="C41" s="3"/>
@@ -2617,7 +1761,7 @@
       <c r="Y41" s="3"/>
       <c r="Z41" s="3"/>
     </row>
-    <row r="42" ht="15.75" customHeight="1" spans="1:26">
+    <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="3"/>
       <c r="B42" s="3"/>
       <c r="C42" s="3"/>
@@ -2645,7 +1789,7 @@
       <c r="Y42" s="3"/>
       <c r="Z42" s="3"/>
     </row>
-    <row r="43" ht="15.75" customHeight="1" spans="1:26">
+    <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="3"/>
       <c r="B43" s="3"/>
       <c r="C43" s="3"/>
@@ -2673,7 +1817,7 @@
       <c r="Y43" s="3"/>
       <c r="Z43" s="3"/>
     </row>
-    <row r="44" ht="15.75" customHeight="1" spans="1:26">
+    <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="3"/>
       <c r="B44" s="3"/>
       <c r="C44" s="3"/>
@@ -2701,7 +1845,7 @@
       <c r="Y44" s="3"/>
       <c r="Z44" s="3"/>
     </row>
-    <row r="45" ht="15.75" customHeight="1" spans="1:26">
+    <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="3"/>
       <c r="B45" s="3"/>
       <c r="C45" s="3"/>
@@ -2729,7 +1873,7 @@
       <c r="Y45" s="3"/>
       <c r="Z45" s="3"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:26">
+    <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="3"/>
       <c r="B46" s="3"/>
       <c r="C46" s="3"/>
@@ -2757,7 +1901,7 @@
       <c r="Y46" s="3"/>
       <c r="Z46" s="3"/>
     </row>
-    <row r="47" ht="15.75" customHeight="1" spans="1:26">
+    <row r="47" ht="15.75" customHeight="1">
       <c r="A47" s="3"/>
       <c r="B47" s="3"/>
       <c r="C47" s="3"/>
@@ -2785,7 +1929,7 @@
       <c r="Y47" s="3"/>
       <c r="Z47" s="3"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:26">
+    <row r="48" ht="15.75" customHeight="1">
       <c r="A48" s="3"/>
       <c r="B48" s="3"/>
       <c r="C48" s="3"/>
@@ -2813,7 +1957,7 @@
       <c r="Y48" s="3"/>
       <c r="Z48" s="3"/>
     </row>
-    <row r="49" ht="15.75" customHeight="1" spans="1:26">
+    <row r="49" ht="15.75" customHeight="1">
       <c r="A49" s="3"/>
       <c r="B49" s="3"/>
       <c r="C49" s="3"/>
@@ -2841,7 +1985,7 @@
       <c r="Y49" s="3"/>
       <c r="Z49" s="3"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:26">
+    <row r="50" ht="15.75" customHeight="1">
       <c r="A50" s="3"/>
       <c r="B50" s="3"/>
       <c r="C50" s="3"/>
@@ -2869,7 +2013,7 @@
       <c r="Y50" s="3"/>
       <c r="Z50" s="3"/>
     </row>
-    <row r="51" ht="15.75" customHeight="1" spans="1:26">
+    <row r="51" ht="15.75" customHeight="1">
       <c r="A51" s="3"/>
       <c r="B51" s="3"/>
       <c r="C51" s="3"/>
@@ -2897,7 +2041,7 @@
       <c r="Y51" s="3"/>
       <c r="Z51" s="3"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:26">
+    <row r="52" ht="15.75" customHeight="1">
       <c r="A52" s="3"/>
       <c r="B52" s="3"/>
       <c r="C52" s="3"/>
@@ -2925,7 +2069,7 @@
       <c r="Y52" s="3"/>
       <c r="Z52" s="3"/>
     </row>
-    <row r="53" ht="15.75" customHeight="1" spans="1:26">
+    <row r="53" ht="15.75" customHeight="1">
       <c r="A53" s="3"/>
       <c r="B53" s="3"/>
       <c r="C53" s="3"/>
@@ -2953,7 +2097,7 @@
       <c r="Y53" s="3"/>
       <c r="Z53" s="3"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:26">
+    <row r="54" ht="15.75" customHeight="1">
       <c r="A54" s="3"/>
       <c r="B54" s="3"/>
       <c r="C54" s="3"/>
@@ -2981,7 +2125,7 @@
       <c r="Y54" s="3"/>
       <c r="Z54" s="3"/>
     </row>
-    <row r="55" ht="15.75" customHeight="1" spans="1:26">
+    <row r="55" ht="15.75" customHeight="1">
       <c r="A55" s="3"/>
       <c r="B55" s="3"/>
       <c r="C55" s="3"/>
@@ -3009,7 +2153,7 @@
       <c r="Y55" s="3"/>
       <c r="Z55" s="3"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:26">
+    <row r="56" ht="15.75" customHeight="1">
       <c r="A56" s="3"/>
       <c r="B56" s="3"/>
       <c r="C56" s="3"/>
@@ -3037,7 +2181,7 @@
       <c r="Y56" s="3"/>
       <c r="Z56" s="3"/>
     </row>
-    <row r="57" ht="15.75" customHeight="1" spans="1:26">
+    <row r="57" ht="15.75" customHeight="1">
       <c r="A57" s="3"/>
       <c r="B57" s="3"/>
       <c r="C57" s="3"/>
@@ -3065,7 +2209,7 @@
       <c r="Y57" s="3"/>
       <c r="Z57" s="3"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:26">
+    <row r="58" ht="15.75" customHeight="1">
       <c r="A58" s="3"/>
       <c r="B58" s="3"/>
       <c r="C58" s="3"/>
@@ -3093,7 +2237,7 @@
       <c r="Y58" s="3"/>
       <c r="Z58" s="3"/>
     </row>
-    <row r="59" ht="15.75" customHeight="1" spans="1:26">
+    <row r="59" ht="15.75" customHeight="1">
       <c r="A59" s="3"/>
       <c r="B59" s="3"/>
       <c r="C59" s="3"/>
@@ -3121,7 +2265,7 @@
       <c r="Y59" s="3"/>
       <c r="Z59" s="3"/>
     </row>
-    <row r="60" ht="15.75" customHeight="1" spans="1:26">
+    <row r="60" ht="15.75" customHeight="1">
       <c r="A60" s="3"/>
       <c r="B60" s="3"/>
       <c r="C60" s="3"/>
@@ -3149,7 +2293,7 @@
       <c r="Y60" s="3"/>
       <c r="Z60" s="3"/>
     </row>
-    <row r="61" ht="15.75" customHeight="1" spans="1:26">
+    <row r="61" ht="15.75" customHeight="1">
       <c r="A61" s="3"/>
       <c r="B61" s="3"/>
       <c r="C61" s="3"/>
@@ -3177,7 +2321,7 @@
       <c r="Y61" s="3"/>
       <c r="Z61" s="3"/>
     </row>
-    <row r="62" ht="15.75" customHeight="1" spans="1:26">
+    <row r="62" ht="15.75" customHeight="1">
       <c r="A62" s="3"/>
       <c r="B62" s="3"/>
       <c r="C62" s="3"/>
@@ -3205,7 +2349,7 @@
       <c r="Y62" s="3"/>
       <c r="Z62" s="3"/>
     </row>
-    <row r="63" ht="15.75" customHeight="1" spans="1:26">
+    <row r="63" ht="15.75" customHeight="1">
       <c r="A63" s="3"/>
       <c r="B63" s="3"/>
       <c r="C63" s="3"/>
@@ -3233,7 +2377,7 @@
       <c r="Y63" s="3"/>
       <c r="Z63" s="3"/>
     </row>
-    <row r="64" ht="15.75" customHeight="1" spans="1:26">
+    <row r="64" ht="15.75" customHeight="1">
       <c r="A64" s="3"/>
       <c r="B64" s="3"/>
       <c r="C64" s="3"/>
@@ -3261,7 +2405,7 @@
       <c r="Y64" s="3"/>
       <c r="Z64" s="3"/>
     </row>
-    <row r="65" ht="15.75" customHeight="1" spans="1:26">
+    <row r="65" ht="15.75" customHeight="1">
       <c r="A65" s="3"/>
       <c r="B65" s="3"/>
       <c r="C65" s="3"/>
@@ -3289,7 +2433,7 @@
       <c r="Y65" s="3"/>
       <c r="Z65" s="3"/>
     </row>
-    <row r="66" ht="15.75" customHeight="1" spans="1:26">
+    <row r="66" ht="15.75" customHeight="1">
       <c r="A66" s="3"/>
       <c r="B66" s="3"/>
       <c r="C66" s="3"/>
@@ -3317,7 +2461,7 @@
       <c r="Y66" s="3"/>
       <c r="Z66" s="3"/>
     </row>
-    <row r="67" ht="15.75" customHeight="1" spans="1:26">
+    <row r="67" ht="15.75" customHeight="1">
       <c r="A67" s="3"/>
       <c r="B67" s="3"/>
       <c r="C67" s="3"/>
@@ -3345,7 +2489,7 @@
       <c r="Y67" s="3"/>
       <c r="Z67" s="3"/>
     </row>
-    <row r="68" ht="15.75" customHeight="1" spans="1:26">
+    <row r="68" ht="15.75" customHeight="1">
       <c r="A68" s="3"/>
       <c r="B68" s="3"/>
       <c r="C68" s="3"/>
@@ -3373,7 +2517,7 @@
       <c r="Y68" s="3"/>
       <c r="Z68" s="3"/>
     </row>
-    <row r="69" ht="15.75" customHeight="1" spans="1:26">
+    <row r="69" ht="15.75" customHeight="1">
       <c r="A69" s="3"/>
       <c r="B69" s="3"/>
       <c r="C69" s="3"/>
@@ -3401,7 +2545,7 @@
       <c r="Y69" s="3"/>
       <c r="Z69" s="3"/>
     </row>
-    <row r="70" ht="15.75" customHeight="1" spans="1:26">
+    <row r="70" ht="15.75" customHeight="1">
       <c r="A70" s="3"/>
       <c r="B70" s="3"/>
       <c r="C70" s="3"/>
@@ -3429,7 +2573,7 @@
       <c r="Y70" s="3"/>
       <c r="Z70" s="3"/>
     </row>
-    <row r="71" ht="15.75" customHeight="1" spans="1:26">
+    <row r="71" ht="15.75" customHeight="1">
       <c r="A71" s="3"/>
       <c r="B71" s="3"/>
       <c r="C71" s="3"/>
@@ -3457,7 +2601,7 @@
       <c r="Y71" s="3"/>
       <c r="Z71" s="3"/>
     </row>
-    <row r="72" ht="15.75" customHeight="1" spans="1:26">
+    <row r="72" ht="15.75" customHeight="1">
       <c r="A72" s="3"/>
       <c r="B72" s="3"/>
       <c r="C72" s="3"/>
@@ -3485,7 +2629,7 @@
       <c r="Y72" s="3"/>
       <c r="Z72" s="3"/>
     </row>
-    <row r="73" ht="15.75" customHeight="1" spans="1:26">
+    <row r="73" ht="15.75" customHeight="1">
       <c r="A73" s="3"/>
       <c r="B73" s="3"/>
       <c r="C73" s="3"/>
@@ -3513,7 +2657,7 @@
       <c r="Y73" s="3"/>
       <c r="Z73" s="3"/>
     </row>
-    <row r="74" ht="15.75" customHeight="1" spans="1:26">
+    <row r="74" ht="15.75" customHeight="1">
       <c r="A74" s="3"/>
       <c r="B74" s="3"/>
       <c r="C74" s="3"/>
@@ -3541,7 +2685,7 @@
       <c r="Y74" s="3"/>
       <c r="Z74" s="3"/>
     </row>
-    <row r="75" ht="15.75" customHeight="1" spans="1:26">
+    <row r="75" ht="15.75" customHeight="1">
       <c r="A75" s="3"/>
       <c r="B75" s="3"/>
       <c r="C75" s="3"/>
@@ -3569,7 +2713,7 @@
       <c r="Y75" s="3"/>
       <c r="Z75" s="3"/>
     </row>
-    <row r="76" ht="15.75" customHeight="1" spans="1:26">
+    <row r="76" ht="15.75" customHeight="1">
       <c r="A76" s="3"/>
       <c r="B76" s="3"/>
       <c r="C76" s="3"/>
@@ -3597,7 +2741,7 @@
       <c r="Y76" s="3"/>
       <c r="Z76" s="3"/>
     </row>
-    <row r="77" ht="15.75" customHeight="1" spans="1:26">
+    <row r="77" ht="15.75" customHeight="1">
       <c r="A77" s="3"/>
       <c r="B77" s="3"/>
       <c r="C77" s="3"/>
@@ -3625,7 +2769,7 @@
       <c r="Y77" s="3"/>
       <c r="Z77" s="3"/>
     </row>
-    <row r="78" ht="15.75" customHeight="1" spans="1:26">
+    <row r="78" ht="15.75" customHeight="1">
       <c r="A78" s="3"/>
       <c r="B78" s="3"/>
       <c r="C78" s="3"/>
@@ -3653,7 +2797,7 @@
       <c r="Y78" s="3"/>
       <c r="Z78" s="3"/>
     </row>
-    <row r="79" ht="15.75" customHeight="1" spans="1:26">
+    <row r="79" ht="15.75" customHeight="1">
       <c r="A79" s="3"/>
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
@@ -3681,7 +2825,7 @@
       <c r="Y79" s="3"/>
       <c r="Z79" s="3"/>
     </row>
-    <row r="80" ht="15.75" customHeight="1" spans="1:26">
+    <row r="80" ht="15.75" customHeight="1">
       <c r="A80" s="3"/>
       <c r="B80" s="3"/>
       <c r="C80" s="3"/>
@@ -3709,7 +2853,7 @@
       <c r="Y80" s="3"/>
       <c r="Z80" s="3"/>
     </row>
-    <row r="81" ht="15.75" customHeight="1" spans="1:26">
+    <row r="81" ht="15.75" customHeight="1">
       <c r="A81" s="3"/>
       <c r="B81" s="3"/>
       <c r="C81" s="3"/>
@@ -3737,7 +2881,7 @@
       <c r="Y81" s="3"/>
       <c r="Z81" s="3"/>
     </row>
-    <row r="82" ht="15.75" customHeight="1" spans="1:26">
+    <row r="82" ht="15.75" customHeight="1">
       <c r="A82" s="3"/>
       <c r="B82" s="3"/>
       <c r="C82" s="3"/>
@@ -3765,7 +2909,7 @@
       <c r="Y82" s="3"/>
       <c r="Z82" s="3"/>
     </row>
-    <row r="83" ht="15.75" customHeight="1" spans="1:26">
+    <row r="83" ht="15.75" customHeight="1">
       <c r="A83" s="3"/>
       <c r="B83" s="3"/>
       <c r="C83" s="3"/>
@@ -3793,7 +2937,7 @@
       <c r="Y83" s="3"/>
       <c r="Z83" s="3"/>
     </row>
-    <row r="84" ht="15.75" customHeight="1" spans="1:26">
+    <row r="84" ht="15.75" customHeight="1">
       <c r="A84" s="3"/>
       <c r="B84" s="3"/>
       <c r="C84" s="3"/>
@@ -3821,7 +2965,7 @@
       <c r="Y84" s="3"/>
       <c r="Z84" s="3"/>
     </row>
-    <row r="85" ht="15.75" customHeight="1" spans="1:26">
+    <row r="85" ht="15.75" customHeight="1">
       <c r="A85" s="3"/>
       <c r="B85" s="3"/>
       <c r="C85" s="3"/>
@@ -3849,7 +2993,7 @@
       <c r="Y85" s="3"/>
       <c r="Z85" s="3"/>
     </row>
-    <row r="86" ht="15.75" customHeight="1" spans="1:26">
+    <row r="86" ht="15.75" customHeight="1">
       <c r="A86" s="3"/>
       <c r="B86" s="3"/>
       <c r="C86" s="3"/>
@@ -3877,7 +3021,7 @@
       <c r="Y86" s="3"/>
       <c r="Z86" s="3"/>
     </row>
-    <row r="87" ht="15.75" customHeight="1" spans="1:26">
+    <row r="87" ht="15.75" customHeight="1">
       <c r="A87" s="3"/>
       <c r="B87" s="3"/>
       <c r="C87" s="3"/>
@@ -3905,7 +3049,7 @@
       <c r="Y87" s="3"/>
       <c r="Z87" s="3"/>
     </row>
-    <row r="88" ht="15.75" customHeight="1" spans="1:26">
+    <row r="88" ht="15.75" customHeight="1">
       <c r="A88" s="3"/>
       <c r="B88" s="3"/>
       <c r="C88" s="3"/>
@@ -3933,7 +3077,7 @@
       <c r="Y88" s="3"/>
       <c r="Z88" s="3"/>
     </row>
-    <row r="89" ht="15.75" customHeight="1" spans="1:26">
+    <row r="89" ht="15.75" customHeight="1">
       <c r="A89" s="3"/>
       <c r="B89" s="3"/>
       <c r="C89" s="3"/>
@@ -3961,7 +3105,7 @@
       <c r="Y89" s="3"/>
       <c r="Z89" s="3"/>
     </row>
-    <row r="90" ht="15.75" customHeight="1" spans="1:26">
+    <row r="90" ht="15.75" customHeight="1">
       <c r="A90" s="3"/>
       <c r="B90" s="3"/>
       <c r="C90" s="3"/>
@@ -3989,7 +3133,7 @@
       <c r="Y90" s="3"/>
       <c r="Z90" s="3"/>
     </row>
-    <row r="91" ht="15.75" customHeight="1" spans="1:26">
+    <row r="91" ht="15.75" customHeight="1">
       <c r="A91" s="3"/>
       <c r="B91" s="3"/>
       <c r="C91" s="3"/>
@@ -4017,7 +3161,7 @@
       <c r="Y91" s="3"/>
       <c r="Z91" s="3"/>
     </row>
-    <row r="92" ht="15.75" customHeight="1" spans="1:26">
+    <row r="92" ht="15.75" customHeight="1">
       <c r="A92" s="3"/>
       <c r="B92" s="3"/>
       <c r="C92" s="3"/>
@@ -4045,7 +3189,7 @@
       <c r="Y92" s="3"/>
       <c r="Z92" s="3"/>
     </row>
-    <row r="93" ht="15.75" customHeight="1" spans="1:26">
+    <row r="93" ht="15.75" customHeight="1">
       <c r="A93" s="3"/>
       <c r="B93" s="3"/>
       <c r="C93" s="3"/>
@@ -4073,7 +3217,7 @@
       <c r="Y93" s="3"/>
       <c r="Z93" s="3"/>
     </row>
-    <row r="94" ht="15.75" customHeight="1" spans="1:26">
+    <row r="94" ht="15.75" customHeight="1">
       <c r="A94" s="3"/>
       <c r="B94" s="3"/>
       <c r="C94" s="3"/>
@@ -4101,7 +3245,7 @@
       <c r="Y94" s="3"/>
       <c r="Z94" s="3"/>
     </row>
-    <row r="95" ht="15.75" customHeight="1" spans="1:26">
+    <row r="95" ht="15.75" customHeight="1">
       <c r="A95" s="3"/>
       <c r="B95" s="3"/>
       <c r="C95" s="3"/>
@@ -4129,7 +3273,7 @@
       <c r="Y95" s="3"/>
       <c r="Z95" s="3"/>
     </row>
-    <row r="96" ht="15.75" customHeight="1" spans="1:26">
+    <row r="96" ht="15.75" customHeight="1">
       <c r="A96" s="3"/>
       <c r="B96" s="3"/>
       <c r="C96" s="3"/>
@@ -4157,7 +3301,7 @@
       <c r="Y96" s="3"/>
       <c r="Z96" s="3"/>
     </row>
-    <row r="97" ht="15.75" customHeight="1" spans="1:26">
+    <row r="97" ht="15.75" customHeight="1">
       <c r="A97" s="3"/>
       <c r="B97" s="3"/>
       <c r="C97" s="3"/>
@@ -4185,7 +3329,7 @@
       <c r="Y97" s="3"/>
       <c r="Z97" s="3"/>
     </row>
-    <row r="98" ht="15.75" customHeight="1" spans="1:26">
+    <row r="98" ht="15.75" customHeight="1">
       <c r="A98" s="3"/>
       <c r="B98" s="3"/>
       <c r="C98" s="3"/>
@@ -4213,7 +3357,7 @@
       <c r="Y98" s="3"/>
       <c r="Z98" s="3"/>
     </row>
-    <row r="99" ht="15.75" customHeight="1" spans="1:26">
+    <row r="99" ht="15.75" customHeight="1">
       <c r="A99" s="3"/>
       <c r="B99" s="3"/>
       <c r="C99" s="3"/>
@@ -4241,7 +3385,7 @@
       <c r="Y99" s="3"/>
       <c r="Z99" s="3"/>
     </row>
-    <row r="100" ht="15.75" customHeight="1" spans="1:26">
+    <row r="100" ht="15.75" customHeight="1">
       <c r="A100" s="3"/>
       <c r="B100" s="3"/>
       <c r="C100" s="3"/>
@@ -4269,7 +3413,7 @@
       <c r="Y100" s="3"/>
       <c r="Z100" s="3"/>
     </row>
-    <row r="101" ht="15.75" customHeight="1" spans="1:26">
+    <row r="101" ht="15.75" customHeight="1">
       <c r="A101" s="3"/>
       <c r="B101" s="3"/>
       <c r="C101" s="3"/>
@@ -4297,7 +3441,7 @@
       <c r="Y101" s="3"/>
       <c r="Z101" s="3"/>
     </row>
-    <row r="102" ht="15.75" customHeight="1" spans="1:26">
+    <row r="102" ht="15.75" customHeight="1">
       <c r="A102" s="3"/>
       <c r="B102" s="3"/>
       <c r="C102" s="3"/>
@@ -4325,7 +3469,7 @@
       <c r="Y102" s="3"/>
       <c r="Z102" s="3"/>
     </row>
-    <row r="103" ht="15.75" customHeight="1" spans="1:26">
+    <row r="103" ht="15.75" customHeight="1">
       <c r="A103" s="3"/>
       <c r="B103" s="3"/>
       <c r="C103" s="3"/>
@@ -4353,7 +3497,7 @@
       <c r="Y103" s="3"/>
       <c r="Z103" s="3"/>
     </row>
-    <row r="104" ht="15.75" customHeight="1" spans="1:26">
+    <row r="104" ht="15.75" customHeight="1">
       <c r="A104" s="3"/>
       <c r="B104" s="3"/>
       <c r="C104" s="3"/>
@@ -4381,7 +3525,7 @@
       <c r="Y104" s="3"/>
       <c r="Z104" s="3"/>
     </row>
-    <row r="105" ht="15.75" customHeight="1" spans="1:26">
+    <row r="105" ht="15.75" customHeight="1">
       <c r="A105" s="3"/>
       <c r="B105" s="3"/>
       <c r="C105" s="3"/>
@@ -4409,7 +3553,7 @@
       <c r="Y105" s="3"/>
       <c r="Z105" s="3"/>
     </row>
-    <row r="106" ht="15.75" customHeight="1" spans="1:26">
+    <row r="106" ht="15.75" customHeight="1">
       <c r="A106" s="3"/>
       <c r="B106" s="3"/>
       <c r="C106" s="3"/>
@@ -4437,7 +3581,7 @@
       <c r="Y106" s="3"/>
       <c r="Z106" s="3"/>
     </row>
-    <row r="107" ht="15.75" customHeight="1" spans="1:26">
+    <row r="107" ht="15.75" customHeight="1">
       <c r="A107" s="3"/>
       <c r="B107" s="3"/>
       <c r="C107" s="3"/>
@@ -4465,7 +3609,7 @@
       <c r="Y107" s="3"/>
       <c r="Z107" s="3"/>
     </row>
-    <row r="108" ht="15.75" customHeight="1" spans="1:26">
+    <row r="108" ht="15.75" customHeight="1">
       <c r="A108" s="3"/>
       <c r="B108" s="3"/>
       <c r="C108" s="3"/>
@@ -4493,7 +3637,7 @@
       <c r="Y108" s="3"/>
       <c r="Z108" s="3"/>
     </row>
-    <row r="109" ht="15.75" customHeight="1" spans="1:26">
+    <row r="109" ht="15.75" customHeight="1">
       <c r="A109" s="3"/>
       <c r="B109" s="3"/>
       <c r="C109" s="3"/>
@@ -4521,7 +3665,7 @@
       <c r="Y109" s="3"/>
       <c r="Z109" s="3"/>
     </row>
-    <row r="110" ht="15.75" customHeight="1" spans="1:26">
+    <row r="110" ht="15.75" customHeight="1">
       <c r="A110" s="3"/>
       <c r="B110" s="3"/>
       <c r="C110" s="3"/>
@@ -4549,7 +3693,7 @@
       <c r="Y110" s="3"/>
       <c r="Z110" s="3"/>
     </row>
-    <row r="111" ht="15.75" customHeight="1" spans="1:26">
+    <row r="111" ht="15.75" customHeight="1">
       <c r="A111" s="3"/>
       <c r="B111" s="3"/>
       <c r="C111" s="3"/>
@@ -4577,7 +3721,7 @@
       <c r="Y111" s="3"/>
       <c r="Z111" s="3"/>
     </row>
-    <row r="112" ht="15.75" customHeight="1" spans="1:26">
+    <row r="112" ht="15.75" customHeight="1">
       <c r="A112" s="3"/>
       <c r="B112" s="3"/>
       <c r="C112" s="3"/>
@@ -4605,7 +3749,7 @@
       <c r="Y112" s="3"/>
       <c r="Z112" s="3"/>
     </row>
-    <row r="113" ht="15.75" customHeight="1" spans="1:26">
+    <row r="113" ht="15.75" customHeight="1">
       <c r="A113" s="3"/>
       <c r="B113" s="3"/>
       <c r="C113" s="3"/>
@@ -4633,7 +3777,7 @@
       <c r="Y113" s="3"/>
       <c r="Z113" s="3"/>
     </row>
-    <row r="114" ht="15.75" customHeight="1" spans="1:26">
+    <row r="114" ht="15.75" customHeight="1">
       <c r="A114" s="3"/>
       <c r="B114" s="3"/>
       <c r="C114" s="3"/>
@@ -4661,7 +3805,7 @@
       <c r="Y114" s="3"/>
       <c r="Z114" s="3"/>
     </row>
-    <row r="115" ht="15.75" customHeight="1" spans="1:26">
+    <row r="115" ht="15.75" customHeight="1">
       <c r="A115" s="3"/>
       <c r="B115" s="3"/>
       <c r="C115" s="3"/>
@@ -4689,7 +3833,7 @@
       <c r="Y115" s="3"/>
       <c r="Z115" s="3"/>
     </row>
-    <row r="116" ht="15.75" customHeight="1" spans="1:26">
+    <row r="116" ht="15.75" customHeight="1">
       <c r="A116" s="3"/>
       <c r="B116" s="3"/>
       <c r="C116" s="3"/>
@@ -4717,7 +3861,7 @@
       <c r="Y116" s="3"/>
       <c r="Z116" s="3"/>
     </row>
-    <row r="117" ht="15.75" customHeight="1" spans="1:26">
+    <row r="117" ht="15.75" customHeight="1">
       <c r="A117" s="3"/>
       <c r="B117" s="3"/>
       <c r="C117" s="3"/>
@@ -4745,7 +3889,7 @@
       <c r="Y117" s="3"/>
       <c r="Z117" s="3"/>
     </row>
-    <row r="118" ht="15.75" customHeight="1" spans="1:26">
+    <row r="118" ht="15.75" customHeight="1">
       <c r="A118" s="3"/>
       <c r="B118" s="3"/>
       <c r="C118" s="3"/>
@@ -4773,7 +3917,7 @@
       <c r="Y118" s="3"/>
       <c r="Z118" s="3"/>
     </row>
-    <row r="119" ht="15.75" customHeight="1" spans="1:26">
+    <row r="119" ht="15.75" customHeight="1">
       <c r="A119" s="3"/>
       <c r="B119" s="3"/>
       <c r="C119" s="3"/>
@@ -4801,7 +3945,7 @@
       <c r="Y119" s="3"/>
       <c r="Z119" s="3"/>
     </row>
-    <row r="120" ht="15.75" customHeight="1" spans="1:26">
+    <row r="120" ht="15.75" customHeight="1">
       <c r="A120" s="3"/>
       <c r="B120" s="3"/>
       <c r="C120" s="3"/>
@@ -4829,7 +3973,7 @@
       <c r="Y120" s="3"/>
       <c r="Z120" s="3"/>
     </row>
-    <row r="121" ht="15.75" customHeight="1" spans="1:26">
+    <row r="121" ht="15.75" customHeight="1">
       <c r="A121" s="3"/>
       <c r="B121" s="3"/>
       <c r="C121" s="3"/>
@@ -4857,7 +4001,7 @@
       <c r="Y121" s="3"/>
       <c r="Z121" s="3"/>
     </row>
-    <row r="122" ht="15.75" customHeight="1" spans="1:26">
+    <row r="122" ht="15.75" customHeight="1">
       <c r="A122" s="3"/>
       <c r="B122" s="3"/>
       <c r="C122" s="3"/>
@@ -4885,7 +4029,7 @@
       <c r="Y122" s="3"/>
       <c r="Z122" s="3"/>
     </row>
-    <row r="123" ht="15.75" customHeight="1" spans="1:26">
+    <row r="123" ht="15.75" customHeight="1">
       <c r="A123" s="3"/>
       <c r="B123" s="3"/>
       <c r="C123" s="3"/>
@@ -4913,7 +4057,7 @@
       <c r="Y123" s="3"/>
       <c r="Z123" s="3"/>
     </row>
-    <row r="124" ht="15.75" customHeight="1" spans="1:26">
+    <row r="124" ht="15.75" customHeight="1">
       <c r="A124" s="3"/>
       <c r="B124" s="3"/>
       <c r="C124" s="3"/>
@@ -4941,7 +4085,7 @@
       <c r="Y124" s="3"/>
       <c r="Z124" s="3"/>
     </row>
-    <row r="125" ht="15.75" customHeight="1" spans="1:26">
+    <row r="125" ht="15.75" customHeight="1">
       <c r="A125" s="3"/>
       <c r="B125" s="3"/>
       <c r="C125" s="3"/>
@@ -4969,7 +4113,7 @@
       <c r="Y125" s="3"/>
       <c r="Z125" s="3"/>
     </row>
-    <row r="126" ht="15.75" customHeight="1" spans="1:26">
+    <row r="126" ht="15.75" customHeight="1">
       <c r="A126" s="3"/>
       <c r="B126" s="3"/>
       <c r="C126" s="3"/>
@@ -4997,7 +4141,7 @@
       <c r="Y126" s="3"/>
       <c r="Z126" s="3"/>
     </row>
-    <row r="127" ht="15.75" customHeight="1" spans="1:26">
+    <row r="127" ht="15.75" customHeight="1">
       <c r="A127" s="3"/>
       <c r="B127" s="3"/>
       <c r="C127" s="3"/>
@@ -5025,7 +4169,7 @@
       <c r="Y127" s="3"/>
       <c r="Z127" s="3"/>
     </row>
-    <row r="128" ht="15.75" customHeight="1" spans="1:26">
+    <row r="128" ht="15.75" customHeight="1">
       <c r="A128" s="3"/>
       <c r="B128" s="3"/>
       <c r="C128" s="3"/>
@@ -5053,7 +4197,7 @@
       <c r="Y128" s="3"/>
       <c r="Z128" s="3"/>
     </row>
-    <row r="129" ht="15.75" customHeight="1" spans="1:26">
+    <row r="129" ht="15.75" customHeight="1">
       <c r="A129" s="3"/>
       <c r="B129" s="3"/>
       <c r="C129" s="3"/>
@@ -5081,7 +4225,7 @@
       <c r="Y129" s="3"/>
       <c r="Z129" s="3"/>
     </row>
-    <row r="130" ht="15.75" customHeight="1" spans="1:26">
+    <row r="130" ht="15.75" customHeight="1">
       <c r="A130" s="3"/>
       <c r="B130" s="3"/>
       <c r="C130" s="3"/>
@@ -5109,7 +4253,7 @@
       <c r="Y130" s="3"/>
       <c r="Z130" s="3"/>
     </row>
-    <row r="131" ht="15.75" customHeight="1" spans="1:26">
+    <row r="131" ht="15.75" customHeight="1">
       <c r="A131" s="3"/>
       <c r="B131" s="3"/>
       <c r="C131" s="3"/>
@@ -5137,7 +4281,7 @@
       <c r="Y131" s="3"/>
       <c r="Z131" s="3"/>
     </row>
-    <row r="132" ht="15.75" customHeight="1" spans="1:26">
+    <row r="132" ht="15.75" customHeight="1">
       <c r="A132" s="3"/>
       <c r="B132" s="3"/>
       <c r="C132" s="3"/>
@@ -5165,7 +4309,7 @@
       <c r="Y132" s="3"/>
       <c r="Z132" s="3"/>
     </row>
-    <row r="133" ht="15.75" customHeight="1" spans="1:26">
+    <row r="133" ht="15.75" customHeight="1">
       <c r="A133" s="3"/>
       <c r="B133" s="3"/>
       <c r="C133" s="3"/>
@@ -5193,7 +4337,7 @@
       <c r="Y133" s="3"/>
       <c r="Z133" s="3"/>
     </row>
-    <row r="134" ht="15.75" customHeight="1" spans="1:26">
+    <row r="134" ht="15.75" customHeight="1">
       <c r="A134" s="3"/>
       <c r="B134" s="3"/>
       <c r="C134" s="3"/>
@@ -5221,7 +4365,7 @@
       <c r="Y134" s="3"/>
       <c r="Z134" s="3"/>
     </row>
-    <row r="135" ht="15.75" customHeight="1" spans="1:26">
+    <row r="135" ht="15.75" customHeight="1">
       <c r="A135" s="3"/>
       <c r="B135" s="3"/>
       <c r="C135" s="3"/>
@@ -5249,7 +4393,7 @@
       <c r="Y135" s="3"/>
       <c r="Z135" s="3"/>
     </row>
-    <row r="136" ht="15.75" customHeight="1" spans="1:26">
+    <row r="136" ht="15.75" customHeight="1">
       <c r="A136" s="3"/>
       <c r="B136" s="3"/>
       <c r="C136" s="3"/>
@@ -5277,7 +4421,7 @@
       <c r="Y136" s="3"/>
       <c r="Z136" s="3"/>
     </row>
-    <row r="137" ht="15.75" customHeight="1" spans="1:26">
+    <row r="137" ht="15.75" customHeight="1">
       <c r="A137" s="3"/>
       <c r="B137" s="3"/>
       <c r="C137" s="3"/>
@@ -5305,7 +4449,7 @@
       <c r="Y137" s="3"/>
       <c r="Z137" s="3"/>
     </row>
-    <row r="138" ht="15.75" customHeight="1" spans="1:26">
+    <row r="138" ht="15.75" customHeight="1">
       <c r="A138" s="3"/>
       <c r="B138" s="3"/>
       <c r="C138" s="3"/>
@@ -5333,7 +4477,7 @@
       <c r="Y138" s="3"/>
       <c r="Z138" s="3"/>
     </row>
-    <row r="139" ht="15.75" customHeight="1" spans="1:26">
+    <row r="139" ht="15.75" customHeight="1">
       <c r="A139" s="3"/>
       <c r="B139" s="3"/>
       <c r="C139" s="3"/>
@@ -5361,7 +4505,7 @@
       <c r="Y139" s="3"/>
       <c r="Z139" s="3"/>
     </row>
-    <row r="140" ht="15.75" customHeight="1" spans="1:26">
+    <row r="140" ht="15.75" customHeight="1">
       <c r="A140" s="3"/>
       <c r="B140" s="3"/>
       <c r="C140" s="3"/>
@@ -5389,7 +4533,7 @@
       <c r="Y140" s="3"/>
       <c r="Z140" s="3"/>
     </row>
-    <row r="141" ht="15.75" customHeight="1" spans="1:26">
+    <row r="141" ht="15.75" customHeight="1">
       <c r="A141" s="3"/>
       <c r="B141" s="3"/>
       <c r="C141" s="3"/>
@@ -5417,7 +4561,7 @@
       <c r="Y141" s="3"/>
       <c r="Z141" s="3"/>
     </row>
-    <row r="142" ht="15.75" customHeight="1" spans="1:26">
+    <row r="142" ht="15.75" customHeight="1">
       <c r="A142" s="3"/>
       <c r="B142" s="3"/>
       <c r="C142" s="3"/>
@@ -5445,7 +4589,7 @@
       <c r="Y142" s="3"/>
       <c r="Z142" s="3"/>
     </row>
-    <row r="143" ht="15.75" customHeight="1" spans="1:26">
+    <row r="143" ht="15.75" customHeight="1">
       <c r="A143" s="3"/>
       <c r="B143" s="3"/>
       <c r="C143" s="3"/>
@@ -5473,7 +4617,7 @@
       <c r="Y143" s="3"/>
       <c r="Z143" s="3"/>
     </row>
-    <row r="144" ht="15.75" customHeight="1" spans="1:26">
+    <row r="144" ht="15.75" customHeight="1">
       <c r="A144" s="3"/>
       <c r="B144" s="3"/>
       <c r="C144" s="3"/>
@@ -5501,7 +4645,7 @@
       <c r="Y144" s="3"/>
       <c r="Z144" s="3"/>
     </row>
-    <row r="145" ht="15.75" customHeight="1" spans="1:26">
+    <row r="145" ht="15.75" customHeight="1">
       <c r="A145" s="3"/>
       <c r="B145" s="3"/>
       <c r="C145" s="3"/>
@@ -5529,7 +4673,7 @@
       <c r="Y145" s="3"/>
       <c r="Z145" s="3"/>
     </row>
-    <row r="146" ht="15.75" customHeight="1" spans="1:26">
+    <row r="146" ht="15.75" customHeight="1">
       <c r="A146" s="3"/>
       <c r="B146" s="3"/>
       <c r="C146" s="3"/>
@@ -5557,7 +4701,7 @@
       <c r="Y146" s="3"/>
       <c r="Z146" s="3"/>
     </row>
-    <row r="147" ht="15.75" customHeight="1" spans="1:26">
+    <row r="147" ht="15.75" customHeight="1">
       <c r="A147" s="3"/>
       <c r="B147" s="3"/>
       <c r="C147" s="3"/>
@@ -5585,7 +4729,7 @@
       <c r="Y147" s="3"/>
       <c r="Z147" s="3"/>
     </row>
-    <row r="148" ht="15.75" customHeight="1" spans="1:26">
+    <row r="148" ht="15.75" customHeight="1">
       <c r="A148" s="3"/>
       <c r="B148" s="3"/>
       <c r="C148" s="3"/>
@@ -5613,7 +4757,7 @@
       <c r="Y148" s="3"/>
       <c r="Z148" s="3"/>
     </row>
-    <row r="149" ht="15.75" customHeight="1" spans="1:26">
+    <row r="149" ht="15.75" customHeight="1">
       <c r="A149" s="3"/>
       <c r="B149" s="3"/>
       <c r="C149" s="3"/>
@@ -5641,7 +4785,7 @@
       <c r="Y149" s="3"/>
       <c r="Z149" s="3"/>
     </row>
-    <row r="150" ht="15.75" customHeight="1" spans="1:26">
+    <row r="150" ht="15.75" customHeight="1">
       <c r="A150" s="3"/>
       <c r="B150" s="3"/>
       <c r="C150" s="3"/>
@@ -5669,7 +4813,7 @@
       <c r="Y150" s="3"/>
       <c r="Z150" s="3"/>
     </row>
-    <row r="151" ht="15.75" customHeight="1" spans="1:26">
+    <row r="151" ht="15.75" customHeight="1">
       <c r="A151" s="3"/>
       <c r="B151" s="3"/>
       <c r="C151" s="3"/>
@@ -5697,7 +4841,7 @@
       <c r="Y151" s="3"/>
       <c r="Z151" s="3"/>
     </row>
-    <row r="152" ht="15.75" customHeight="1" spans="1:26">
+    <row r="152" ht="15.75" customHeight="1">
       <c r="A152" s="3"/>
       <c r="B152" s="3"/>
       <c r="C152" s="3"/>
@@ -5725,7 +4869,7 @@
       <c r="Y152" s="3"/>
       <c r="Z152" s="3"/>
     </row>
-    <row r="153" ht="15.75" customHeight="1" spans="1:26">
+    <row r="153" ht="15.75" customHeight="1">
       <c r="A153" s="3"/>
       <c r="B153" s="3"/>
       <c r="C153" s="3"/>
@@ -5753,7 +4897,7 @@
       <c r="Y153" s="3"/>
       <c r="Z153" s="3"/>
     </row>
-    <row r="154" ht="15.75" customHeight="1" spans="1:26">
+    <row r="154" ht="15.75" customHeight="1">
       <c r="A154" s="3"/>
       <c r="B154" s="3"/>
       <c r="C154" s="3"/>
@@ -5781,7 +4925,7 @@
       <c r="Y154" s="3"/>
       <c r="Z154" s="3"/>
     </row>
-    <row r="155" ht="15.75" customHeight="1" spans="1:26">
+    <row r="155" ht="15.75" customHeight="1">
       <c r="A155" s="3"/>
       <c r="B155" s="3"/>
       <c r="C155" s="3"/>
@@ -5809,7 +4953,7 @@
       <c r="Y155" s="3"/>
       <c r="Z155" s="3"/>
     </row>
-    <row r="156" ht="15.75" customHeight="1" spans="1:26">
+    <row r="156" ht="15.75" customHeight="1">
       <c r="A156" s="3"/>
       <c r="B156" s="3"/>
       <c r="C156" s="3"/>
@@ -5837,7 +4981,7 @@
       <c r="Y156" s="3"/>
       <c r="Z156" s="3"/>
     </row>
-    <row r="157" ht="15.75" customHeight="1" spans="1:26">
+    <row r="157" ht="15.75" customHeight="1">
       <c r="A157" s="3"/>
       <c r="B157" s="3"/>
       <c r="C157" s="3"/>
@@ -5865,7 +5009,7 @@
       <c r="Y157" s="3"/>
       <c r="Z157" s="3"/>
     </row>
-    <row r="158" ht="15.75" customHeight="1" spans="1:26">
+    <row r="158" ht="15.75" customHeight="1">
       <c r="A158" s="3"/>
       <c r="B158" s="3"/>
       <c r="C158" s="3"/>
@@ -5893,7 +5037,7 @@
       <c r="Y158" s="3"/>
       <c r="Z158" s="3"/>
     </row>
-    <row r="159" ht="15.75" customHeight="1" spans="1:26">
+    <row r="159" ht="15.75" customHeight="1">
       <c r="A159" s="3"/>
       <c r="B159" s="3"/>
       <c r="C159" s="3"/>
@@ -5921,7 +5065,7 @@
       <c r="Y159" s="3"/>
       <c r="Z159" s="3"/>
     </row>
-    <row r="160" ht="15.75" customHeight="1" spans="1:26">
+    <row r="160" ht="15.75" customHeight="1">
       <c r="A160" s="3"/>
       <c r="B160" s="3"/>
       <c r="C160" s="3"/>
@@ -5949,7 +5093,7 @@
       <c r="Y160" s="3"/>
       <c r="Z160" s="3"/>
     </row>
-    <row r="161" ht="15.75" customHeight="1" spans="1:26">
+    <row r="161" ht="15.75" customHeight="1">
       <c r="A161" s="3"/>
       <c r="B161" s="3"/>
       <c r="C161" s="3"/>
@@ -5977,7 +5121,7 @@
       <c r="Y161" s="3"/>
       <c r="Z161" s="3"/>
     </row>
-    <row r="162" ht="15.75" customHeight="1" spans="1:26">
+    <row r="162" ht="15.75" customHeight="1">
       <c r="A162" s="3"/>
       <c r="B162" s="3"/>
       <c r="C162" s="3"/>
@@ -6005,7 +5149,7 @@
       <c r="Y162" s="3"/>
       <c r="Z162" s="3"/>
     </row>
-    <row r="163" ht="15.75" customHeight="1" spans="1:26">
+    <row r="163" ht="15.75" customHeight="1">
       <c r="A163" s="3"/>
       <c r="B163" s="3"/>
       <c r="C163" s="3"/>
@@ -6033,7 +5177,7 @@
       <c r="Y163" s="3"/>
       <c r="Z163" s="3"/>
     </row>
-    <row r="164" ht="15.75" customHeight="1" spans="1:26">
+    <row r="164" ht="15.75" customHeight="1">
       <c r="A164" s="3"/>
       <c r="B164" s="3"/>
       <c r="C164" s="3"/>
@@ -6061,7 +5205,7 @@
       <c r="Y164" s="3"/>
       <c r="Z164" s="3"/>
     </row>
-    <row r="165" ht="15.75" customHeight="1" spans="1:26">
+    <row r="165" ht="15.75" customHeight="1">
       <c r="A165" s="3"/>
       <c r="B165" s="3"/>
       <c r="C165" s="3"/>
@@ -6089,7 +5233,7 @@
       <c r="Y165" s="3"/>
       <c r="Z165" s="3"/>
     </row>
-    <row r="166" ht="15.75" customHeight="1" spans="1:26">
+    <row r="166" ht="15.75" customHeight="1">
       <c r="A166" s="3"/>
       <c r="B166" s="3"/>
       <c r="C166" s="3"/>
@@ -6117,7 +5261,7 @@
       <c r="Y166" s="3"/>
       <c r="Z166" s="3"/>
     </row>
-    <row r="167" ht="15.75" customHeight="1" spans="1:26">
+    <row r="167" ht="15.75" customHeight="1">
       <c r="A167" s="3"/>
       <c r="B167" s="3"/>
       <c r="C167" s="3"/>
@@ -6145,7 +5289,7 @@
       <c r="Y167" s="3"/>
       <c r="Z167" s="3"/>
     </row>
-    <row r="168" ht="15.75" customHeight="1" spans="1:26">
+    <row r="168" ht="15.75" customHeight="1">
       <c r="A168" s="3"/>
       <c r="B168" s="3"/>
       <c r="C168" s="3"/>
@@ -6173,7 +5317,7 @@
       <c r="Y168" s="3"/>
       <c r="Z168" s="3"/>
     </row>
-    <row r="169" ht="15.75" customHeight="1" spans="1:26">
+    <row r="169" ht="15.75" customHeight="1">
       <c r="A169" s="3"/>
       <c r="B169" s="3"/>
       <c r="C169" s="3"/>
@@ -6201,7 +5345,7 @@
       <c r="Y169" s="3"/>
       <c r="Z169" s="3"/>
     </row>
-    <row r="170" ht="15.75" customHeight="1" spans="1:26">
+    <row r="170" ht="15.75" customHeight="1">
       <c r="A170" s="3"/>
       <c r="B170" s="3"/>
       <c r="C170" s="3"/>
@@ -6229,7 +5373,7 @@
       <c r="Y170" s="3"/>
       <c r="Z170" s="3"/>
     </row>
-    <row r="171" ht="15.75" customHeight="1" spans="1:26">
+    <row r="171" ht="15.75" customHeight="1">
       <c r="A171" s="3"/>
       <c r="B171" s="3"/>
       <c r="C171" s="3"/>
@@ -6257,7 +5401,7 @@
       <c r="Y171" s="3"/>
       <c r="Z171" s="3"/>
     </row>
-    <row r="172" ht="15.75" customHeight="1" spans="1:26">
+    <row r="172" ht="15.75" customHeight="1">
       <c r="A172" s="3"/>
       <c r="B172" s="3"/>
       <c r="C172" s="3"/>
@@ -6285,7 +5429,7 @@
       <c r="Y172" s="3"/>
       <c r="Z172" s="3"/>
     </row>
-    <row r="173" ht="15.75" customHeight="1" spans="1:26">
+    <row r="173" ht="15.75" customHeight="1">
       <c r="A173" s="3"/>
       <c r="B173" s="3"/>
       <c r="C173" s="3"/>
@@ -6313,7 +5457,7 @@
       <c r="Y173" s="3"/>
       <c r="Z173" s="3"/>
     </row>
-    <row r="174" ht="15.75" customHeight="1" spans="1:26">
+    <row r="174" ht="15.75" customHeight="1">
       <c r="A174" s="3"/>
       <c r="B174" s="3"/>
       <c r="C174" s="3"/>
@@ -6341,7 +5485,7 @@
       <c r="Y174" s="3"/>
       <c r="Z174" s="3"/>
     </row>
-    <row r="175" ht="15.75" customHeight="1" spans="1:26">
+    <row r="175" ht="15.75" customHeight="1">
       <c r="A175" s="3"/>
       <c r="B175" s="3"/>
       <c r="C175" s="3"/>
@@ -6369,7 +5513,7 @@
       <c r="Y175" s="3"/>
       <c r="Z175" s="3"/>
     </row>
-    <row r="176" ht="15.75" customHeight="1" spans="1:26">
+    <row r="176" ht="15.75" customHeight="1">
       <c r="A176" s="3"/>
       <c r="B176" s="3"/>
       <c r="C176" s="3"/>
@@ -6397,7 +5541,7 @@
       <c r="Y176" s="3"/>
       <c r="Z176" s="3"/>
     </row>
-    <row r="177" ht="15.75" customHeight="1" spans="1:26">
+    <row r="177" ht="15.75" customHeight="1">
       <c r="A177" s="3"/>
       <c r="B177" s="3"/>
       <c r="C177" s="3"/>
@@ -6425,7 +5569,7 @@
       <c r="Y177" s="3"/>
       <c r="Z177" s="3"/>
     </row>
-    <row r="178" ht="15.75" customHeight="1" spans="1:26">
+    <row r="178" ht="15.75" customHeight="1">
       <c r="A178" s="3"/>
       <c r="B178" s="3"/>
       <c r="C178" s="3"/>
@@ -6453,7 +5597,7 @@
       <c r="Y178" s="3"/>
       <c r="Z178" s="3"/>
     </row>
-    <row r="179" ht="15.75" customHeight="1" spans="1:26">
+    <row r="179" ht="15.75" customHeight="1">
       <c r="A179" s="3"/>
       <c r="B179" s="3"/>
       <c r="C179" s="3"/>
@@ -6481,7 +5625,7 @@
       <c r="Y179" s="3"/>
       <c r="Z179" s="3"/>
     </row>
-    <row r="180" ht="15.75" customHeight="1" spans="1:26">
+    <row r="180" ht="15.75" customHeight="1">
       <c r="A180" s="3"/>
       <c r="B180" s="3"/>
       <c r="C180" s="3"/>
@@ -6509,7 +5653,7 @@
       <c r="Y180" s="3"/>
       <c r="Z180" s="3"/>
     </row>
-    <row r="181" ht="15.75" customHeight="1" spans="1:26">
+    <row r="181" ht="15.75" customHeight="1">
       <c r="A181" s="3"/>
       <c r="B181" s="3"/>
       <c r="C181" s="3"/>
@@ -6537,7 +5681,7 @@
       <c r="Y181" s="3"/>
       <c r="Z181" s="3"/>
     </row>
-    <row r="182" ht="15.75" customHeight="1" spans="1:26">
+    <row r="182" ht="15.75" customHeight="1">
       <c r="A182" s="3"/>
       <c r="B182" s="3"/>
       <c r="C182" s="3"/>
@@ -6565,7 +5709,7 @@
       <c r="Y182" s="3"/>
       <c r="Z182" s="3"/>
     </row>
-    <row r="183" ht="15.75" customHeight="1" spans="1:26">
+    <row r="183" ht="15.75" customHeight="1">
       <c r="A183" s="3"/>
       <c r="B183" s="3"/>
       <c r="C183" s="3"/>
@@ -6593,7 +5737,7 @@
       <c r="Y183" s="3"/>
       <c r="Z183" s="3"/>
     </row>
-    <row r="184" ht="15.75" customHeight="1" spans="1:26">
+    <row r="184" ht="15.75" customHeight="1">
       <c r="A184" s="3"/>
       <c r="B184" s="3"/>
       <c r="C184" s="3"/>
@@ -6621,7 +5765,7 @@
       <c r="Y184" s="3"/>
       <c r="Z184" s="3"/>
     </row>
-    <row r="185" ht="15.75" customHeight="1" spans="1:26">
+    <row r="185" ht="15.75" customHeight="1">
       <c r="A185" s="3"/>
       <c r="B185" s="3"/>
       <c r="C185" s="3"/>
@@ -6649,7 +5793,7 @@
       <c r="Y185" s="3"/>
       <c r="Z185" s="3"/>
     </row>
-    <row r="186" ht="15.75" customHeight="1" spans="1:26">
+    <row r="186" ht="15.75" customHeight="1">
       <c r="A186" s="3"/>
       <c r="B186" s="3"/>
       <c r="C186" s="3"/>
@@ -6677,7 +5821,7 @@
       <c r="Y186" s="3"/>
       <c r="Z186" s="3"/>
     </row>
-    <row r="187" ht="15.75" customHeight="1" spans="1:26">
+    <row r="187" ht="15.75" customHeight="1">
       <c r="A187" s="3"/>
       <c r="B187" s="3"/>
       <c r="C187" s="3"/>
@@ -6705,7 +5849,7 @@
       <c r="Y187" s="3"/>
       <c r="Z187" s="3"/>
     </row>
-    <row r="188" ht="15.75" customHeight="1" spans="1:26">
+    <row r="188" ht="15.75" customHeight="1">
       <c r="A188" s="3"/>
       <c r="B188" s="3"/>
       <c r="C188" s="3"/>
@@ -6733,7 +5877,7 @@
       <c r="Y188" s="3"/>
       <c r="Z188" s="3"/>
     </row>
-    <row r="189" ht="15.75" customHeight="1" spans="1:26">
+    <row r="189" ht="15.75" customHeight="1">
       <c r="A189" s="3"/>
       <c r="B189" s="3"/>
       <c r="C189" s="3"/>
@@ -6761,7 +5905,7 @@
       <c r="Y189" s="3"/>
       <c r="Z189" s="3"/>
     </row>
-    <row r="190" ht="15.75" customHeight="1" spans="1:26">
+    <row r="190" ht="15.75" customHeight="1">
       <c r="A190" s="3"/>
       <c r="B190" s="3"/>
       <c r="C190" s="3"/>
@@ -6789,7 +5933,7 @@
       <c r="Y190" s="3"/>
       <c r="Z190" s="3"/>
     </row>
-    <row r="191" ht="15.75" customHeight="1" spans="1:26">
+    <row r="191" ht="15.75" customHeight="1">
       <c r="A191" s="3"/>
       <c r="B191" s="3"/>
       <c r="C191" s="3"/>
@@ -6817,7 +5961,7 @@
       <c r="Y191" s="3"/>
       <c r="Z191" s="3"/>
     </row>
-    <row r="192" ht="15.75" customHeight="1" spans="1:26">
+    <row r="192" ht="15.75" customHeight="1">
       <c r="A192" s="3"/>
       <c r="B192" s="3"/>
       <c r="C192" s="3"/>
@@ -6845,7 +5989,7 @@
       <c r="Y192" s="3"/>
       <c r="Z192" s="3"/>
     </row>
-    <row r="193" ht="15.75" customHeight="1" spans="1:26">
+    <row r="193" ht="15.75" customHeight="1">
       <c r="A193" s="3"/>
       <c r="B193" s="3"/>
       <c r="C193" s="3"/>
@@ -6873,7 +6017,7 @@
       <c r="Y193" s="3"/>
       <c r="Z193" s="3"/>
     </row>
-    <row r="194" ht="15.75" customHeight="1" spans="1:26">
+    <row r="194" ht="15.75" customHeight="1">
       <c r="A194" s="3"/>
       <c r="B194" s="3"/>
       <c r="C194" s="3"/>
@@ -6901,7 +6045,7 @@
       <c r="Y194" s="3"/>
       <c r="Z194" s="3"/>
     </row>
-    <row r="195" ht="15.75" customHeight="1" spans="1:26">
+    <row r="195" ht="15.75" customHeight="1">
       <c r="A195" s="3"/>
       <c r="B195" s="3"/>
       <c r="C195" s="3"/>
@@ -6929,7 +6073,7 @@
       <c r="Y195" s="3"/>
       <c r="Z195" s="3"/>
     </row>
-    <row r="196" ht="15.75" customHeight="1" spans="1:26">
+    <row r="196" ht="15.75" customHeight="1">
       <c r="A196" s="3"/>
       <c r="B196" s="3"/>
       <c r="C196" s="3"/>
@@ -6957,7 +6101,7 @@
       <c r="Y196" s="3"/>
       <c r="Z196" s="3"/>
     </row>
-    <row r="197" ht="15.75" customHeight="1" spans="1:26">
+    <row r="197" ht="15.75" customHeight="1">
       <c r="A197" s="3"/>
       <c r="B197" s="3"/>
       <c r="C197" s="3"/>
@@ -6985,7 +6129,7 @@
       <c r="Y197" s="3"/>
       <c r="Z197" s="3"/>
     </row>
-    <row r="198" ht="15.75" customHeight="1" spans="1:26">
+    <row r="198" ht="15.75" customHeight="1">
       <c r="A198" s="3"/>
       <c r="B198" s="3"/>
       <c r="C198" s="3"/>
@@ -7013,7 +6157,7 @@
       <c r="Y198" s="3"/>
       <c r="Z198" s="3"/>
     </row>
-    <row r="199" ht="15.75" customHeight="1" spans="1:26">
+    <row r="199" ht="15.75" customHeight="1">
       <c r="A199" s="3"/>
       <c r="B199" s="3"/>
       <c r="C199" s="3"/>
@@ -7041,7 +6185,7 @@
       <c r="Y199" s="3"/>
       <c r="Z199" s="3"/>
     </row>
-    <row r="200" ht="15.75" customHeight="1" spans="1:26">
+    <row r="200" ht="15.75" customHeight="1">
       <c r="A200" s="3"/>
       <c r="B200" s="3"/>
       <c r="C200" s="3"/>
@@ -7069,7 +6213,7 @@
       <c r="Y200" s="3"/>
       <c r="Z200" s="3"/>
     </row>
-    <row r="201" ht="15.75" customHeight="1" spans="1:26">
+    <row r="201" ht="15.75" customHeight="1">
       <c r="A201" s="3"/>
       <c r="B201" s="3"/>
       <c r="C201" s="3"/>
@@ -7097,7 +6241,7 @@
       <c r="Y201" s="3"/>
       <c r="Z201" s="3"/>
     </row>
-    <row r="202" ht="15.75" customHeight="1" spans="1:26">
+    <row r="202" ht="15.75" customHeight="1">
       <c r="A202" s="3"/>
       <c r="B202" s="3"/>
       <c r="C202" s="3"/>
@@ -7125,7 +6269,7 @@
       <c r="Y202" s="3"/>
       <c r="Z202" s="3"/>
     </row>
-    <row r="203" ht="15.75" customHeight="1" spans="1:26">
+    <row r="203" ht="15.75" customHeight="1">
       <c r="A203" s="3"/>
       <c r="B203" s="3"/>
       <c r="C203" s="3"/>
@@ -7153,7 +6297,7 @@
       <c r="Y203" s="3"/>
       <c r="Z203" s="3"/>
     </row>
-    <row r="204" ht="15.75" customHeight="1" spans="1:26">
+    <row r="204" ht="15.75" customHeight="1">
       <c r="A204" s="3"/>
       <c r="B204" s="3"/>
       <c r="C204" s="3"/>
@@ -7181,7 +6325,7 @@
       <c r="Y204" s="3"/>
       <c r="Z204" s="3"/>
     </row>
-    <row r="205" ht="15.75" customHeight="1" spans="1:26">
+    <row r="205" ht="15.75" customHeight="1">
       <c r="A205" s="3"/>
       <c r="B205" s="3"/>
       <c r="C205" s="3"/>
@@ -7209,7 +6353,7 @@
       <c r="Y205" s="3"/>
       <c r="Z205" s="3"/>
     </row>
-    <row r="206" ht="15.75" customHeight="1" spans="1:26">
+    <row r="206" ht="15.75" customHeight="1">
       <c r="A206" s="3"/>
       <c r="B206" s="3"/>
       <c r="C206" s="3"/>
@@ -7237,7 +6381,7 @@
       <c r="Y206" s="3"/>
       <c r="Z206" s="3"/>
     </row>
-    <row r="207" ht="15.75" customHeight="1" spans="1:26">
+    <row r="207" ht="15.75" customHeight="1">
       <c r="A207" s="3"/>
       <c r="B207" s="3"/>
       <c r="C207" s="3"/>
@@ -7265,7 +6409,7 @@
       <c r="Y207" s="3"/>
       <c r="Z207" s="3"/>
     </row>
-    <row r="208" ht="15.75" customHeight="1" spans="1:26">
+    <row r="208" ht="15.75" customHeight="1">
       <c r="A208" s="3"/>
       <c r="B208" s="3"/>
       <c r="C208" s="3"/>
@@ -7293,7 +6437,7 @@
       <c r="Y208" s="3"/>
       <c r="Z208" s="3"/>
     </row>
-    <row r="209" ht="15.75" customHeight="1" spans="1:26">
+    <row r="209" ht="15.75" customHeight="1">
       <c r="A209" s="3"/>
       <c r="B209" s="3"/>
       <c r="C209" s="3"/>
@@ -7321,7 +6465,7 @@
       <c r="Y209" s="3"/>
       <c r="Z209" s="3"/>
     </row>
-    <row r="210" ht="15.75" customHeight="1" spans="1:26">
+    <row r="210" ht="15.75" customHeight="1">
       <c r="A210" s="3"/>
       <c r="B210" s="3"/>
       <c r="C210" s="3"/>
@@ -7349,7 +6493,7 @@
       <c r="Y210" s="3"/>
       <c r="Z210" s="3"/>
     </row>
-    <row r="211" ht="15.75" customHeight="1" spans="1:26">
+    <row r="211" ht="15.75" customHeight="1">
       <c r="A211" s="3"/>
       <c r="B211" s="3"/>
       <c r="C211" s="3"/>
@@ -7377,7 +6521,7 @@
       <c r="Y211" s="3"/>
       <c r="Z211" s="3"/>
     </row>
-    <row r="212" ht="15.75" customHeight="1" spans="1:26">
+    <row r="212" ht="15.75" customHeight="1">
       <c r="A212" s="3"/>
       <c r="B212" s="3"/>
       <c r="C212" s="3"/>
@@ -7405,7 +6549,7 @@
       <c r="Y212" s="3"/>
       <c r="Z212" s="3"/>
     </row>
-    <row r="213" ht="15.75" customHeight="1" spans="1:26">
+    <row r="213" ht="15.75" customHeight="1">
       <c r="A213" s="3"/>
       <c r="B213" s="3"/>
       <c r="C213" s="3"/>
@@ -7433,7 +6577,7 @@
       <c r="Y213" s="3"/>
       <c r="Z213" s="3"/>
     </row>
-    <row r="214" ht="15.75" customHeight="1" spans="1:26">
+    <row r="214" ht="15.75" customHeight="1">
       <c r="A214" s="3"/>
       <c r="B214" s="3"/>
       <c r="C214" s="3"/>
@@ -7461,7 +6605,7 @@
       <c r="Y214" s="3"/>
       <c r="Z214" s="3"/>
     </row>
-    <row r="215" ht="15.75" customHeight="1" spans="1:26">
+    <row r="215" ht="15.75" customHeight="1">
       <c r="A215" s="3"/>
       <c r="B215" s="3"/>
       <c r="C215" s="3"/>
@@ -7489,7 +6633,7 @@
       <c r="Y215" s="3"/>
       <c r="Z215" s="3"/>
     </row>
-    <row r="216" ht="15.75" customHeight="1" spans="1:26">
+    <row r="216" ht="15.75" customHeight="1">
       <c r="A216" s="3"/>
       <c r="B216" s="3"/>
       <c r="C216" s="3"/>
@@ -7517,7 +6661,7 @@
       <c r="Y216" s="3"/>
       <c r="Z216" s="3"/>
     </row>
-    <row r="217" ht="15.75" customHeight="1" spans="1:26">
+    <row r="217" ht="15.75" customHeight="1">
       <c r="A217" s="3"/>
       <c r="B217" s="3"/>
       <c r="C217" s="3"/>
@@ -7545,7 +6689,7 @@
       <c r="Y217" s="3"/>
       <c r="Z217" s="3"/>
     </row>
-    <row r="218" ht="15.75" customHeight="1" spans="1:26">
+    <row r="218" ht="15.75" customHeight="1">
       <c r="A218" s="3"/>
       <c r="B218" s="3"/>
       <c r="C218" s="3"/>
@@ -7573,7 +6717,7 @@
       <c r="Y218" s="3"/>
       <c r="Z218" s="3"/>
     </row>
-    <row r="219" ht="15.75" customHeight="1" spans="1:26">
+    <row r="219" ht="15.75" customHeight="1">
       <c r="A219" s="3"/>
       <c r="B219" s="3"/>
       <c r="C219" s="3"/>
@@ -7601,7 +6745,7 @@
       <c r="Y219" s="3"/>
       <c r="Z219" s="3"/>
     </row>
-    <row r="220" ht="15.75" customHeight="1" spans="1:26">
+    <row r="220" ht="15.75" customHeight="1">
       <c r="A220" s="3"/>
       <c r="B220" s="3"/>
       <c r="C220" s="3"/>
@@ -8410,8 +7554,9 @@
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
-  <pageMargins left="0.699999988079071" right="0.699999988079071" top="0.75" bottom="0.75" header="0" footer="0"/>
+  <printOptions/>
+  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.699999988079071" right="0.699999988079071" top="0.75"/>
   <pageSetup paperSize="9" orientation="portrait"/>
-  <headerFooter/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat/refactor: PlayerInventory 관련 리팩토링
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/ItemData.xlsx
+++ b/JsonConverter/ExcelFiles/ItemData.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="149">
   <si>
     <t>아이템 ID</t>
   </si>
@@ -96,7 +96,10 @@
     <t>Husks</t>
   </si>
   <si>
-    <t>HoldType</t>
+    <t>StringHoldType</t>
+  </si>
+  <si>
+    <t>MeshCollider</t>
   </si>
   <si>
     <t>Item_Tool_MasterKey</t>
@@ -112,7 +115,7 @@
     <t>Tool</t>
   </si>
   <si>
-    <t>None</t>
+    <t>Epic</t>
   </si>
   <si>
     <t>Yellow</t>
@@ -121,7 +124,10 @@
     <t>KeyFBX[SM_Gen_Prop_Key_01]</t>
   </si>
   <si>
-    <t>ToolObject</t>
+    <t>Pool_Tool</t>
+  </si>
+  <si>
+    <t>Hold</t>
   </si>
   <si>
     <t>Item_Tool_Key</t>
@@ -134,6 +140,9 @@
 한 번만 사용 할 수 있다.</t>
   </si>
   <si>
+    <t>Rare</t>
+  </si>
+  <si>
     <t>Black</t>
   </si>
   <si>
@@ -149,19 +158,13 @@
     <t>Jewel</t>
   </si>
   <si>
-    <t>Epic</t>
-  </si>
-  <si>
     <t>M_Gemstone_Diamond,Lit</t>
   </si>
   <si>
     <t>Jewel_Cone[Cone]</t>
   </si>
   <si>
-    <t>JewelObject</t>
-  </si>
-  <si>
-    <t>Hold</t>
+    <t>Pool_Jewel</t>
   </si>
   <si>
     <t>Item_Jewel_Amethyst</t>
@@ -203,9 +206,6 @@
     <t>에메랄드다.</t>
   </si>
   <si>
-    <t>Rare</t>
-  </si>
-  <si>
     <t>M_Gemstone_Emerald</t>
   </si>
   <si>
@@ -360,6 +360,111 @@
   </si>
   <si>
     <t>Statue_Marble</t>
+  </si>
+  <si>
+    <t>Item_Junk_Bottle_Blue</t>
+  </si>
+  <si>
+    <t>파란 병</t>
+  </si>
+  <si>
+    <t>평범한 파란 병이다.</t>
+  </si>
+  <si>
+    <t>Junk</t>
+  </si>
+  <si>
+    <t>PolygonNightclubs_01_A</t>
+  </si>
+  <si>
+    <t>Junk_Bottle_Blue[SM_Prop_Bar_Bottle_07]</t>
+  </si>
+  <si>
+    <t>JunkObject</t>
+  </si>
+  <si>
+    <t>MeshCollider_Junk_Bottle_Blue</t>
+  </si>
+  <si>
+    <t>Item_Junk_Bottle_Pink_Large</t>
+  </si>
+  <si>
+    <t>큰 핑크색 병</t>
+  </si>
+  <si>
+    <t>크기가 큰 핑크색 병이다.</t>
+  </si>
+  <si>
+    <t>Junk_Bottle_Pink_Large[SM_Prop_Bottle_Large_01]</t>
+  </si>
+  <si>
+    <t>MeshCollider_Junk_Bottle_Pink_Large</t>
+  </si>
+  <si>
+    <t>Item_Junk_Can_Navy</t>
+  </si>
+  <si>
+    <t>남색 캔</t>
+  </si>
+  <si>
+    <t>누가 먹다남은 음료이다.</t>
+  </si>
+  <si>
+    <t>Junk_Can_Navy[SM_Prop_Can_01]</t>
+  </si>
+  <si>
+    <t>Item_Junk_Fish</t>
+  </si>
+  <si>
+    <t>청새치</t>
+  </si>
+  <si>
+    <t>엄청 큰 청새치다. 맛있어 보인다.</t>
+  </si>
+  <si>
+    <t>Junk_Fish[SM_Prop_Display_Fish_02]</t>
+  </si>
+  <si>
+    <t>Item_Junk_Glasses</t>
+  </si>
+  <si>
+    <t>썬글라스</t>
+  </si>
+  <si>
+    <t>화려한 썬글라스다.</t>
+  </si>
+  <si>
+    <t>Junk_Glasses[SM_Prop_Glasses_01]</t>
+  </si>
+  <si>
+    <t>MeshCollider_Junk_Glasses</t>
+  </si>
+  <si>
+    <t>Item_Junk_Microphone</t>
+  </si>
+  <si>
+    <t>마이크</t>
+  </si>
+  <si>
+    <t>손 마이크이다.</t>
+  </si>
+  <si>
+    <t>Junk_Microphone[SM_Prop_Microphone_01]</t>
+  </si>
+  <si>
+    <t>Item_Junk_Sculpture</t>
+  </si>
+  <si>
+    <t>조각품</t>
+  </si>
+  <si>
+    <t>예술가의 혼이 담긴 조각품이다.</t>
+  </si>
+  <si>
+    <t>PolygonNightclub_Mat_01_A_Metallic,PolygonNightclubs_01_A</t>
+  </si>
+  <si>
+    <t>Junk_Sculpture[SM_Prop_Sculpture_01]</t>
   </si>
 </sst>
 </file>
@@ -719,16 +824,17 @@
     <col customWidth="1" min="1" max="1" width="25.38"/>
     <col customWidth="1" min="2" max="2" width="15.0"/>
     <col customWidth="1" min="3" max="3" width="24.25"/>
-    <col customWidth="1" min="4" max="4" width="15.5"/>
-    <col customWidth="1" min="5" max="5" width="14.5"/>
+    <col customWidth="1" min="4" max="4" width="12.75"/>
+    <col customWidth="1" min="5" max="5" width="13.25"/>
     <col customWidth="1" min="6" max="6" width="11.63"/>
     <col customWidth="1" min="7" max="7" width="9.63"/>
-    <col customWidth="1" min="8" max="8" width="23.75"/>
-    <col customWidth="1" min="9" max="9" width="14.13"/>
+    <col customWidth="1" min="8" max="8" width="9.38"/>
+    <col customWidth="1" min="9" max="9" width="8.63"/>
     <col customWidth="1" min="10" max="10" width="21.25"/>
-    <col customWidth="1" min="11" max="11" width="27.38"/>
+    <col customWidth="1" min="11" max="11" width="28.38"/>
     <col customWidth="1" min="12" max="12" width="11.75"/>
-    <col customWidth="1" min="13" max="21" width="9.63"/>
+    <col customWidth="1" min="13" max="13" width="16.13"/>
+    <col customWidth="1" min="14" max="21" width="9.63"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
@@ -814,7 +920,9 @@
       <c r="M2" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="N2" s="4"/>
+      <c r="N2" s="3" t="s">
+        <v>10</v>
+      </c>
       <c r="O2" s="4"/>
       <c r="P2" s="4"/>
       <c r="Q2" s="4"/>
@@ -863,7 +971,9 @@
       <c r="M3" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="N3" s="10"/>
+      <c r="N3" s="9" t="s">
+        <v>27</v>
+      </c>
       <c r="O3" s="10"/>
       <c r="P3" s="10"/>
       <c r="Q3" s="10"/>
@@ -874,19 +984,19 @@
     </row>
     <row r="4" ht="15.0" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F4" s="4">
         <v>2.0</v>
@@ -899,15 +1009,17 @@
         <v>-1.0</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="L4" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="M4" s="4"/>
+      <c r="L4" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="M4" s="11" t="s">
+        <v>36</v>
+      </c>
       <c r="N4" s="4"/>
       <c r="O4" s="4"/>
       <c r="P4" s="4"/>
@@ -919,19 +1031,19 @@
     </row>
     <row r="5" ht="15.0" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="F5" s="4">
         <v>1.0</v>
@@ -944,15 +1056,17 @@
         <v>1.0</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="K5" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="L5" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="M5" s="4"/>
+      <c r="L5" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="M5" s="11" t="s">
+        <v>36</v>
+      </c>
       <c r="N5" s="4"/>
       <c r="O5" s="4"/>
       <c r="P5" s="4"/>
@@ -964,19 +1078,19 @@
     </row>
     <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="6" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="F6" s="4">
         <v>10.0</v>
@@ -987,16 +1101,16 @@
       <c r="H6" s="4"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="L6" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>48</v>
       </c>
       <c r="M6" s="11" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="N6" s="4"/>
       <c r="O6" s="4"/>
@@ -1009,19 +1123,19 @@
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="F7" s="4">
         <v>8.0</v>
@@ -1032,16 +1146,16 @@
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="K7" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="L7" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
+      </c>
+      <c r="L7" s="3" t="s">
+        <v>48</v>
       </c>
       <c r="M7" s="11" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="N7" s="4"/>
       <c r="O7" s="4"/>
@@ -1054,19 +1168,19 @@
     </row>
     <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F8" s="4">
         <v>7.0</v>
@@ -1077,16 +1191,16 @@
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="K8" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="L8" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
+      </c>
+      <c r="L8" s="3" t="s">
+        <v>48</v>
       </c>
       <c r="M8" s="11" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="N8" s="4"/>
       <c r="O8" s="4"/>
@@ -1099,19 +1213,19 @@
     </row>
     <row r="9" ht="15.75" customHeight="1">
       <c r="A9" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>61</v>
+        <v>32</v>
       </c>
       <c r="F9" s="4">
         <v>6.0</v>
@@ -1125,13 +1239,13 @@
         <v>62</v>
       </c>
       <c r="K9" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="L9" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
+      </c>
+      <c r="L9" s="3" t="s">
+        <v>48</v>
       </c>
       <c r="M9" s="11" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="N9" s="4"/>
       <c r="O9" s="4"/>
@@ -1153,10 +1267,10 @@
         <v>65</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="F10" s="4">
         <v>5.0</v>
@@ -1170,13 +1284,13 @@
         <v>66</v>
       </c>
       <c r="K10" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="L10" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
+      </c>
+      <c r="L10" s="3" t="s">
+        <v>48</v>
       </c>
       <c r="M10" s="11" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="N10" s="4"/>
       <c r="O10" s="4"/>
@@ -1198,7 +1312,7 @@
         <v>69</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>70</v>
@@ -1215,13 +1329,13 @@
         <v>71</v>
       </c>
       <c r="K11" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="L11" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
+      </c>
+      <c r="L11" s="3" t="s">
+        <v>48</v>
       </c>
       <c r="M11" s="11" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="N11" s="4"/>
       <c r="O11" s="4"/>
@@ -1243,7 +1357,7 @@
         <v>74</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>70</v>
@@ -1260,13 +1374,13 @@
         <v>75</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="L12" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
+      </c>
+      <c r="L12" s="3" t="s">
+        <v>48</v>
       </c>
       <c r="M12" s="11" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="N12" s="4"/>
       <c r="O12" s="4"/>
@@ -1291,7 +1405,7 @@
         <v>79</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="F13" s="14">
         <v>12.0</v>
@@ -1311,7 +1425,7 @@
         <v>82</v>
       </c>
       <c r="M13" s="13" t="s">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="N13" s="15"/>
       <c r="O13" s="15"/>
@@ -1336,7 +1450,7 @@
         <v>79</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="F14" s="14">
         <v>12.0</v>
@@ -1356,7 +1470,7 @@
         <v>82</v>
       </c>
       <c r="M14" s="13" t="s">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="N14" s="15"/>
       <c r="O14" s="15"/>
@@ -1381,7 +1495,7 @@
         <v>79</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="F15" s="14">
         <v>12.0</v>
@@ -1401,7 +1515,7 @@
         <v>82</v>
       </c>
       <c r="M15" s="13" t="s">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="N15" s="15"/>
       <c r="O15" s="15"/>
@@ -1426,7 +1540,7 @@
         <v>79</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="F16" s="14">
         <v>12.0</v>
@@ -1446,7 +1560,7 @@
         <v>82</v>
       </c>
       <c r="M16" s="13" t="s">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="N16" s="15"/>
       <c r="O16" s="15"/>
@@ -1471,7 +1585,7 @@
         <v>79</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="F17" s="14">
         <v>12.0</v>
@@ -1491,7 +1605,7 @@
         <v>82</v>
       </c>
       <c r="M17" s="13" t="s">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="N17" s="15"/>
       <c r="O17" s="15"/>
@@ -1516,7 +1630,7 @@
         <v>98</v>
       </c>
       <c r="E18" s="13" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="F18" s="14">
         <v>5.0</v>
@@ -1536,7 +1650,7 @@
         <v>101</v>
       </c>
       <c r="M18" s="13" t="s">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="N18" s="4"/>
       <c r="O18" s="4"/>
@@ -1561,7 +1675,7 @@
         <v>98</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="F19" s="14">
         <v>10.0</v>
@@ -1581,7 +1695,7 @@
         <v>101</v>
       </c>
       <c r="M19" s="13" t="s">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="N19" s="4"/>
       <c r="O19" s="4"/>
@@ -1606,7 +1720,7 @@
         <v>98</v>
       </c>
       <c r="E20" s="13" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F20" s="14">
         <v>15.0</v>
@@ -1626,7 +1740,7 @@
         <v>101</v>
       </c>
       <c r="M20" s="13" t="s">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="N20" s="4"/>
       <c r="O20" s="4"/>
@@ -1671,7 +1785,7 @@
         <v>101</v>
       </c>
       <c r="M21" s="13" t="s">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="N21" s="4"/>
       <c r="O21" s="4"/>
@@ -1683,20 +1797,42 @@
       <c r="U21" s="4"/>
     </row>
     <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="4"/>
-      <c r="B22" s="4"/>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
+      <c r="A22" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F22" s="14">
+        <v>5.0</v>
+      </c>
+      <c r="G22" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H22" s="4"/>
       <c r="I22" s="4"/>
-      <c r="J22" s="4"/>
-      <c r="K22" s="4"/>
-      <c r="L22" s="4"/>
+      <c r="J22" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="K22" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="L22" s="3" t="s">
+        <v>120</v>
+      </c>
       <c r="M22" s="4"/>
-      <c r="N22" s="4"/>
+      <c r="N22" s="3" t="s">
+        <v>121</v>
+      </c>
       <c r="O22" s="4"/>
       <c r="P22" s="4"/>
       <c r="Q22" s="4"/>
@@ -1706,20 +1842,42 @@
       <c r="U22" s="4"/>
     </row>
     <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="4"/>
-      <c r="B23" s="4"/>
-      <c r="C23" s="4"/>
-      <c r="D23" s="4"/>
-      <c r="E23" s="4"/>
-      <c r="F23" s="4"/>
-      <c r="G23" s="4"/>
+      <c r="A23" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F23" s="14">
+        <v>5.0</v>
+      </c>
+      <c r="G23" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H23" s="4"/>
       <c r="I23" s="4"/>
-      <c r="J23" s="4"/>
-      <c r="K23" s="4"/>
-      <c r="L23" s="4"/>
+      <c r="J23" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="K23" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="L23" s="3" t="s">
+        <v>120</v>
+      </c>
       <c r="M23" s="4"/>
-      <c r="N23" s="4"/>
+      <c r="N23" s="3" t="s">
+        <v>126</v>
+      </c>
       <c r="O23" s="4"/>
       <c r="P23" s="4"/>
       <c r="Q23" s="4"/>
@@ -1729,18 +1887,38 @@
       <c r="U23" s="4"/>
     </row>
     <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="4"/>
-      <c r="B24" s="4"/>
-      <c r="C24" s="4"/>
-      <c r="D24" s="4"/>
-      <c r="E24" s="4"/>
-      <c r="F24" s="4"/>
-      <c r="G24" s="4"/>
+      <c r="A24" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F24" s="14">
+        <v>5.0</v>
+      </c>
+      <c r="G24" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H24" s="4"/>
       <c r="I24" s="4"/>
-      <c r="J24" s="4"/>
-      <c r="K24" s="4"/>
-      <c r="L24" s="4"/>
+      <c r="J24" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="K24" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="L24" s="3" t="s">
+        <v>120</v>
+      </c>
       <c r="M24" s="4"/>
       <c r="N24" s="4"/>
       <c r="O24" s="4"/>
@@ -1752,19 +1930,41 @@
       <c r="U24" s="4"/>
     </row>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="4"/>
-      <c r="B25" s="4"/>
-      <c r="C25" s="4"/>
-      <c r="D25" s="4"/>
-      <c r="E25" s="4"/>
-      <c r="F25" s="4"/>
-      <c r="G25" s="4"/>
+      <c r="A25" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="E25" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="F25" s="14">
+        <v>15.0</v>
+      </c>
+      <c r="G25" s="14">
+        <v>4000.0</v>
+      </c>
       <c r="H25" s="4"/>
       <c r="I25" s="4"/>
-      <c r="J25" s="4"/>
-      <c r="K25" s="4"/>
-      <c r="L25" s="4"/>
-      <c r="M25" s="4"/>
+      <c r="J25" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="K25" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="L25" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="M25" s="13" t="s">
+        <v>36</v>
+      </c>
       <c r="N25" s="4"/>
       <c r="O25" s="4"/>
       <c r="P25" s="4"/>
@@ -1775,20 +1975,42 @@
       <c r="U25" s="4"/>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="4"/>
-      <c r="B26" s="4"/>
-      <c r="C26" s="4"/>
-      <c r="D26" s="4"/>
-      <c r="E26" s="4"/>
-      <c r="F26" s="4"/>
-      <c r="G26" s="4"/>
+      <c r="A26" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F26" s="14">
+        <v>5.0</v>
+      </c>
+      <c r="G26" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H26" s="4"/>
       <c r="I26" s="4"/>
-      <c r="J26" s="4"/>
-      <c r="K26" s="4"/>
-      <c r="L26" s="4"/>
+      <c r="J26" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="K26" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="L26" s="3" t="s">
+        <v>120</v>
+      </c>
       <c r="M26" s="4"/>
-      <c r="N26" s="4"/>
+      <c r="N26" s="3" t="s">
+        <v>139</v>
+      </c>
       <c r="O26" s="4"/>
       <c r="P26" s="4"/>
       <c r="Q26" s="4"/>
@@ -1798,17 +2020,35 @@
       <c r="U26" s="4"/>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="4"/>
-      <c r="B27" s="4"/>
-      <c r="C27" s="4"/>
-      <c r="D27" s="4"/>
-      <c r="E27" s="4"/>
-      <c r="F27" s="4"/>
-      <c r="G27" s="4"/>
+      <c r="A27" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F27" s="14">
+        <v>5.0</v>
+      </c>
+      <c r="G27" s="3">
+        <v>100.0</v>
+      </c>
       <c r="H27" s="4"/>
       <c r="I27" s="4"/>
-      <c r="J27" s="4"/>
-      <c r="K27" s="4"/>
+      <c r="J27" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="K27" s="3" t="s">
+        <v>143</v>
+      </c>
       <c r="L27" s="4"/>
       <c r="M27" s="4"/>
       <c r="N27" s="4"/>
@@ -1821,17 +2061,35 @@
       <c r="U27" s="4"/>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="4"/>
-      <c r="B28" s="4"/>
-      <c r="C28" s="4"/>
-      <c r="D28" s="4"/>
-      <c r="E28" s="4"/>
-      <c r="F28" s="4"/>
-      <c r="G28" s="4"/>
+      <c r="A28" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="E28" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="F28" s="14">
+        <v>20.0</v>
+      </c>
+      <c r="G28" s="14">
+        <v>5000.0</v>
+      </c>
       <c r="H28" s="4"/>
       <c r="I28" s="4"/>
-      <c r="J28" s="4"/>
-      <c r="K28" s="4"/>
+      <c r="J28" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="K28" s="3" t="s">
+        <v>148</v>
+      </c>
       <c r="L28" s="4"/>
       <c r="M28" s="4"/>
       <c r="N28" s="4"/>

</xml_diff>